<commit_message>
atualização do anexo A
</commit_message>
<xml_diff>
--- a/Anexo A.xlsx
+++ b/Anexo A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\ADM -POLI\CoC\Engenharia Eletrônica 2027\Ementas Oficial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C6D4F27-163F-4100-99D5-F66CCCCFD2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7962B87A-17D0-499B-8655-16F6F61EA3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="215">
   <si>
     <t>Código</t>
   </si>
@@ -596,50 +596,6 @@
     <t xml:space="preserve">Antenas, Micro-ondas e Óptica Moderna </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Informações específicas:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Para a conclusão do Curso, o aluno deverá cursar:
-1) Todas as disciplinas solicitadas na grade curricular do 1º ao 10º semestres, (obrigatórias, eletivas e livres) considerando inclusive todas as informações específicas;
-2) No 8º semestre, o aluno deverá cursar 12 créditos de um conjunto de cinco disciplinas optativas eletivas do curso.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">3) No 9º semestre e no 10º semestre,  o aluno deverá cursar 24 créditos de disciplinas optativas eletivas do curso.
-</t>
-    </r>
-  </si>
-  <si>
     <t>2000201</t>
   </si>
   <si>
@@ -707,6 +663,55 @@
   </si>
   <si>
     <t>PSI0322 (forte)</t>
+  </si>
+  <si>
+    <t>Fundamentos de Adaptação e Aprendizado de Máquina</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Informações específicas:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Para a conclusão do Curso, o aluno deverá cursar:
+1) Todas as disciplinas solicitadas na grade curricular do 1º ao 10º semestres, (obrigatórias, eletivas e livres) considerando inclusive todas as informações específicas;
+2) No 8º semestre, o aluno deverá cursar 12 créditos de um conjunto de cinco disciplinas optativas eletivas do curso.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3) No 9º semestre e no 10º semestre,  o aluno deverá cursar 24 créditos de disciplinas optativas eletivas do curso.
+4) 60 horas, i.e., 2 créditos trabalho de AAC (Atividades Acadêmicas Complementares) para a conclusão do curso. Os créditos podem ser obtidos em qualquer semestre do curso, e por isso não estão representados na tabela. Ainda, o aluno poderá obter créditos trabalho de AAC adicionais, mas limitado ao total de 12 créditos trabalho (360 horas). As atividades aceitas como AAC, os créditos trabalho atribuídos a cada atividade, e a forma de comprovação da execução da atividade estão descritas em regulamento definido pela Comissão de Graduação e são válidas e comuns para todos os cursos da EPUSP.
+5) O aluno deverá cursar obrigatoriamente até o final de seu curso um total de 480 horas em Atividades Extensionistas Curriculares (AEX). Os créditos de AEX são integralmente integralizados com as disciplinas de Projeto Integrativo. 
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1366,7 +1371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="196">
+  <cellXfs count="195">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1656,9 +1661,6 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1740,8 +1742,26 @@
     <xf numFmtId="3" fontId="17" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1752,8 +1772,47 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1764,98 +1823,38 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="13" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1896,61 +1895,64 @@
     <xf numFmtId="3" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2258,36 +2260,36 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Z990"/>
+  <dimension ref="A1:Z988"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" style="98" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" style="97" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="55.109375" style="72" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" style="98" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="97" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" style="72" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.6640625" style="98" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="5.44140625" style="98" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.6640625" style="98" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.44140625" style="98" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" style="97" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="5.44140625" style="97" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.6640625" style="97" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.44140625" style="97" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.109375" style="72" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="8.6640625" style="72" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="41.44140625" style="72" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="8.6640625" style="98" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="8.6640625" style="97" bestFit="1" customWidth="1"/>
     <col min="16" max="26" width="8.6640625" style="72" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="124" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="192"/>
-      <c r="C1" s="193"/>
-      <c r="D1" s="192"/>
-      <c r="E1" s="193"/>
-      <c r="F1" s="193"/>
-      <c r="G1" s="193"/>
-      <c r="H1" s="193"/>
-      <c r="I1" s="194"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="127"/>
       <c r="J1" s="25"/>
       <c r="K1" s="26"/>
       <c r="L1" s="26"/>
@@ -2314,10 +2316,10 @@
       <c r="E2" s="30"/>
       <c r="F2" s="30"/>
       <c r="G2" s="30"/>
-      <c r="H2" s="195" t="s">
+      <c r="H2" s="128" t="s">
         <v>72</v>
       </c>
-      <c r="I2" s="145"/>
+      <c r="I2" s="129"/>
       <c r="J2" s="25"/>
       <c r="K2" s="26"/>
       <c r="L2" s="26"/>
@@ -2337,17 +2339,17 @@
       <c r="Z2" s="26"/>
     </row>
     <row r="3" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="135" t="s">
+      <c r="A3" s="130" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="126"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="128"/>
+      <c r="B3" s="131"/>
+      <c r="C3" s="132"/>
+      <c r="D3" s="131"/>
+      <c r="E3" s="132"/>
+      <c r="F3" s="132"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="132"/>
+      <c r="I3" s="133"/>
       <c r="J3" s="25"/>
       <c r="K3" s="26"/>
       <c r="L3" s="26"/>
@@ -2367,17 +2369,17 @@
       <c r="Z3" s="26"/>
     </row>
     <row r="4" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="133" t="s">
+      <c r="A4" s="134" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="126"/>
-      <c r="C4" s="127"/>
-      <c r="D4" s="126"/>
-      <c r="E4" s="127"/>
-      <c r="F4" s="127"/>
-      <c r="G4" s="127"/>
-      <c r="H4" s="127"/>
-      <c r="I4" s="128"/>
+      <c r="B4" s="131"/>
+      <c r="C4" s="132"/>
+      <c r="D4" s="131"/>
+      <c r="E4" s="132"/>
+      <c r="F4" s="132"/>
+      <c r="G4" s="132"/>
+      <c r="H4" s="132"/>
+      <c r="I4" s="133"/>
       <c r="J4" s="25"/>
       <c r="K4" s="26"/>
       <c r="L4" s="26"/>
@@ -2406,11 +2408,11 @@
       </c>
       <c r="D5" s="35"/>
       <c r="E5" s="34"/>
-      <c r="F5" s="188" t="s">
+      <c r="F5" s="135" t="s">
         <v>77</v>
       </c>
-      <c r="G5" s="127"/>
-      <c r="H5" s="183"/>
+      <c r="G5" s="132"/>
+      <c r="H5" s="136"/>
       <c r="I5" s="36" t="s">
         <v>78</v>
       </c>
@@ -2440,11 +2442,11 @@
       <c r="C6" s="34"/>
       <c r="D6" s="35"/>
       <c r="E6" s="34"/>
-      <c r="F6" s="188" t="s">
+      <c r="F6" s="135" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="127"/>
-      <c r="H6" s="183"/>
+      <c r="G6" s="132"/>
+      <c r="H6" s="136"/>
       <c r="I6" s="36" t="s">
         <v>78</v>
       </c>
@@ -2468,17 +2470,17 @@
     </row>
     <row r="7" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="32" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="34"/>
       <c r="D7" s="35"/>
       <c r="E7" s="34"/>
-      <c r="F7" s="188" t="s">
+      <c r="F7" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="G7" s="127"/>
-      <c r="H7" s="183"/>
+      <c r="G7" s="132"/>
+      <c r="H7" s="136"/>
       <c r="I7" s="36" t="s">
         <v>82</v>
       </c>
@@ -2531,15 +2533,15 @@
       <c r="Z8" s="26"/>
     </row>
     <row r="9" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="189"/>
-      <c r="B9" s="126"/>
-      <c r="C9" s="127"/>
-      <c r="D9" s="126"/>
-      <c r="E9" s="127"/>
-      <c r="F9" s="127"/>
-      <c r="G9" s="127"/>
-      <c r="H9" s="127"/>
-      <c r="I9" s="128"/>
+      <c r="A9" s="137"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="132"/>
+      <c r="D9" s="131"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="132"/>
+      <c r="H9" s="132"/>
+      <c r="I9" s="133"/>
       <c r="J9" s="26"/>
       <c r="K9" s="26"/>
       <c r="L9" s="26"/>
@@ -2559,23 +2561,23 @@
       <c r="Z9" s="26"/>
     </row>
     <row r="10" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="189" t="s">
+      <c r="A10" s="137" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="156"/>
-      <c r="C10" s="178" t="s">
+      <c r="B10" s="138"/>
+      <c r="C10" s="139" t="s">
         <v>85</v>
       </c>
-      <c r="D10" s="180" t="s">
+      <c r="D10" s="141" t="s">
         <v>86</v>
       </c>
-      <c r="E10" s="182" t="s">
+      <c r="E10" s="143" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="127"/>
-      <c r="G10" s="127"/>
-      <c r="H10" s="183"/>
-      <c r="I10" s="184" t="s">
+      <c r="F10" s="132"/>
+      <c r="G10" s="132"/>
+      <c r="H10" s="136"/>
+      <c r="I10" s="144" t="s">
         <v>88</v>
       </c>
       <c r="J10" s="39"/>
@@ -2597,12 +2599,12 @@
       <c r="Z10" s="26"/>
     </row>
     <row r="11" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="190" t="s">
+      <c r="A11" s="146" t="s">
         <v>89</v>
       </c>
-      <c r="B11" s="156"/>
-      <c r="C11" s="179"/>
-      <c r="D11" s="181"/>
+      <c r="B11" s="138"/>
+      <c r="C11" s="140"/>
+      <c r="D11" s="142"/>
       <c r="E11" s="40" t="s">
         <v>90</v>
       </c>
@@ -2615,7 +2617,7 @@
       <c r="H11" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="I11" s="185"/>
+      <c r="I11" s="145"/>
       <c r="J11" s="39"/>
       <c r="K11" s="26"/>
       <c r="L11" s="26"/>
@@ -2635,17 +2637,17 @@
       <c r="Z11" s="26"/>
     </row>
     <row r="12" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="186" t="s">
+      <c r="A12" s="147" t="s">
         <v>94</v>
       </c>
-      <c r="B12" s="130"/>
-      <c r="C12" s="131"/>
-      <c r="D12" s="130"/>
-      <c r="E12" s="131"/>
-      <c r="F12" s="131"/>
-      <c r="G12" s="131"/>
-      <c r="H12" s="131"/>
-      <c r="I12" s="132"/>
+      <c r="B12" s="148"/>
+      <c r="C12" s="149"/>
+      <c r="D12" s="148"/>
+      <c r="E12" s="149"/>
+      <c r="F12" s="149"/>
+      <c r="G12" s="149"/>
+      <c r="H12" s="149"/>
+      <c r="I12" s="150"/>
       <c r="J12" s="39"/>
       <c r="K12" s="26"/>
       <c r="L12" s="26"/>
@@ -2665,26 +2667,26 @@
       <c r="Z12" s="26"/>
     </row>
     <row r="13" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="107" t="s">
+      <c r="A13" s="106" t="s">
         <v>95</v>
       </c>
-      <c r="B13" s="100" t="s">
+      <c r="B13" s="99" t="s">
         <v>96</v>
       </c>
-      <c r="C13" s="101"/>
-      <c r="D13" s="100"/>
-      <c r="E13" s="102">
+      <c r="C13" s="100"/>
+      <c r="D13" s="99"/>
+      <c r="E13" s="101">
         <v>4</v>
       </c>
-      <c r="F13" s="102">
+      <c r="F13" s="101">
         <v>4</v>
       </c>
-      <c r="G13" s="102"/>
-      <c r="H13" s="102">
+      <c r="G13" s="101"/>
+      <c r="H13" s="101">
         <f>SUM(E13:F13)</f>
         <v>8</v>
       </c>
-      <c r="I13" s="103">
+      <c r="I13" s="102">
         <f>E13*15+F13*30</f>
         <v>180</v>
       </c>
@@ -2707,24 +2709,24 @@
       <c r="Z13" s="26"/>
     </row>
     <row r="14" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="109" t="s">
-        <v>191</v>
-      </c>
-      <c r="B14" s="100" t="s">
+      <c r="A14" s="108" t="s">
+        <v>190</v>
+      </c>
+      <c r="B14" s="99" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="101"/>
-      <c r="D14" s="100"/>
-      <c r="E14" s="102">
+      <c r="C14" s="100"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="101">
         <v>10</v>
       </c>
-      <c r="F14" s="102"/>
-      <c r="G14" s="102"/>
-      <c r="H14" s="102">
+      <c r="F14" s="101"/>
+      <c r="G14" s="101"/>
+      <c r="H14" s="101">
         <f>SUM(E14:F14)</f>
         <v>10</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <f>E14*15+F14*30</f>
         <v>150</v>
       </c>
@@ -2747,24 +2749,24 @@
       <c r="Z14" s="26"/>
     </row>
     <row r="15" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="107" t="s">
+      <c r="A15" s="106" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="100" t="s">
-        <v>193</v>
-      </c>
-      <c r="C15" s="101"/>
-      <c r="D15" s="100"/>
-      <c r="E15" s="102">
+      <c r="B15" s="99" t="s">
+        <v>192</v>
+      </c>
+      <c r="C15" s="100"/>
+      <c r="D15" s="99"/>
+      <c r="E15" s="101">
         <v>4</v>
       </c>
-      <c r="F15" s="102"/>
-      <c r="G15" s="102"/>
-      <c r="H15" s="102">
+      <c r="F15" s="101"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="101">
         <f>SUM(E15:F15)</f>
         <v>4</v>
       </c>
-      <c r="I15" s="103">
+      <c r="I15" s="102">
         <f>E15*15+F15*30</f>
         <v>60</v>
       </c>
@@ -2787,24 +2789,24 @@
       <c r="Z15" s="26"/>
     </row>
     <row r="16" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="107" t="s">
-        <v>195</v>
-      </c>
-      <c r="B16" s="100" t="s">
+      <c r="A16" s="106" t="s">
+        <v>194</v>
+      </c>
+      <c r="B16" s="99" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="101"/>
-      <c r="D16" s="100"/>
-      <c r="E16" s="102">
+      <c r="C16" s="100"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="101">
         <v>3</v>
       </c>
-      <c r="F16" s="102"/>
-      <c r="G16" s="102"/>
-      <c r="H16" s="102">
+      <c r="F16" s="101"/>
+      <c r="G16" s="101"/>
+      <c r="H16" s="101">
         <f>SUM(E16:F16)</f>
         <v>3</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <f>E16*15+F16*30</f>
         <v>45</v>
       </c>
@@ -2827,24 +2829,24 @@
       <c r="Z16" s="26"/>
     </row>
     <row r="17" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="107" t="s">
+      <c r="A17" s="106" t="s">
         <v>100</v>
       </c>
-      <c r="B17" s="100" t="s">
+      <c r="B17" s="99" t="s">
         <v>101</v>
       </c>
-      <c r="C17" s="101"/>
-      <c r="D17" s="100"/>
-      <c r="E17" s="102">
+      <c r="C17" s="100"/>
+      <c r="D17" s="99"/>
+      <c r="E17" s="101">
         <v>3</v>
       </c>
-      <c r="F17" s="102"/>
-      <c r="G17" s="102"/>
-      <c r="H17" s="102">
+      <c r="F17" s="101"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="101">
         <f>SUM(E17:F17)</f>
         <v>3</v>
       </c>
-      <c r="I17" s="103">
+      <c r="I17" s="102">
         <f>E17*15+F17*30</f>
         <v>45</v>
       </c>
@@ -2867,29 +2869,29 @@
       <c r="Z17" s="26"/>
     </row>
     <row r="18" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="99"/>
-      <c r="B18" s="161" t="s">
+      <c r="A18" s="98"/>
+      <c r="B18" s="151" t="s">
         <v>102</v>
       </c>
-      <c r="C18" s="159"/>
-      <c r="D18" s="162"/>
-      <c r="E18" s="104">
+      <c r="C18" s="152"/>
+      <c r="D18" s="153"/>
+      <c r="E18" s="103">
         <f>SUM(E13:E17)</f>
         <v>24</v>
       </c>
-      <c r="F18" s="104">
+      <c r="F18" s="103">
         <f>SUM(F13:F17)</f>
         <v>4</v>
       </c>
-      <c r="G18" s="104">
+      <c r="G18" s="103">
         <f>SUM(G13:G17)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="104">
+      <c r="H18" s="103">
         <f>SUM(H13:H17)</f>
         <v>28</v>
       </c>
-      <c r="I18" s="105">
+      <c r="I18" s="104">
         <f>SUM(I13:I17)</f>
         <v>480</v>
       </c>
@@ -2912,15 +2914,15 @@
       <c r="Z18" s="26"/>
     </row>
     <row r="19" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="163"/>
-      <c r="B19" s="158"/>
-      <c r="C19" s="159"/>
-      <c r="D19" s="158"/>
-      <c r="E19" s="159"/>
-      <c r="F19" s="159"/>
-      <c r="G19" s="159"/>
-      <c r="H19" s="159"/>
-      <c r="I19" s="160"/>
+      <c r="A19" s="154"/>
+      <c r="B19" s="155"/>
+      <c r="C19" s="152"/>
+      <c r="D19" s="155"/>
+      <c r="E19" s="152"/>
+      <c r="F19" s="152"/>
+      <c r="G19" s="152"/>
+      <c r="H19" s="152"/>
+      <c r="I19" s="156"/>
       <c r="J19" s="39"/>
       <c r="K19" s="26"/>
       <c r="L19" s="26"/>
@@ -2940,17 +2942,17 @@
       <c r="Z19" s="26"/>
     </row>
     <row r="20" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="187" t="s">
+      <c r="A20" s="157" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="158"/>
-      <c r="C20" s="159"/>
-      <c r="D20" s="158"/>
-      <c r="E20" s="159"/>
-      <c r="F20" s="159"/>
-      <c r="G20" s="159"/>
-      <c r="H20" s="159"/>
-      <c r="I20" s="160"/>
+      <c r="B20" s="155"/>
+      <c r="C20" s="152"/>
+      <c r="D20" s="155"/>
+      <c r="E20" s="152"/>
+      <c r="F20" s="152"/>
+      <c r="G20" s="152"/>
+      <c r="H20" s="152"/>
+      <c r="I20" s="156"/>
       <c r="J20" s="39"/>
       <c r="K20" s="26"/>
       <c r="L20" s="26"/>
@@ -2970,28 +2972,28 @@
       <c r="Z20" s="26"/>
     </row>
     <row r="21" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="107" t="s">
+      <c r="A21" s="106" t="s">
         <v>104</v>
       </c>
-      <c r="B21" s="100" t="s">
+      <c r="B21" s="99" t="s">
         <v>105</v>
       </c>
-      <c r="C21" s="101"/>
-      <c r="D21" s="100"/>
-      <c r="E21" s="102">
+      <c r="C21" s="100"/>
+      <c r="D21" s="99"/>
+      <c r="E21" s="101">
         <v>4</v>
       </c>
-      <c r="F21" s="102">
+      <c r="F21" s="101">
         <v>4</v>
       </c>
-      <c r="G21" s="102">
+      <c r="G21" s="101">
         <v>4</v>
       </c>
-      <c r="H21" s="102">
+      <c r="H21" s="101">
         <f>SUM(E21:F21)</f>
         <v>8</v>
       </c>
-      <c r="I21" s="103">
+      <c r="I21" s="102">
         <f>E21*15+F21*30</f>
         <v>180</v>
       </c>
@@ -3014,24 +3016,24 @@
       <c r="Z21" s="26"/>
     </row>
     <row r="22" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="109" t="s">
-        <v>192</v>
-      </c>
-      <c r="B22" s="100" t="s">
+      <c r="A22" s="108" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" s="99" t="s">
         <v>106</v>
       </c>
-      <c r="C22" s="101"/>
-      <c r="D22" s="100"/>
-      <c r="E22" s="102">
+      <c r="C22" s="100"/>
+      <c r="D22" s="99"/>
+      <c r="E22" s="101">
         <v>10</v>
       </c>
-      <c r="F22" s="102"/>
-      <c r="G22" s="102"/>
-      <c r="H22" s="102">
+      <c r="F22" s="101"/>
+      <c r="G22" s="101"/>
+      <c r="H22" s="101">
         <f>SUM(E22:F22)</f>
         <v>10</v>
       </c>
-      <c r="I22" s="103">
+      <c r="I22" s="102">
         <f>E22*15+F22*30</f>
         <v>150</v>
       </c>
@@ -3054,24 +3056,24 @@
       <c r="Z22" s="26"/>
     </row>
     <row r="23" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="107" t="s">
+      <c r="A23" s="106" t="s">
         <v>107</v>
       </c>
-      <c r="B23" s="100" t="s">
-        <v>194</v>
-      </c>
-      <c r="C23" s="101"/>
-      <c r="D23" s="100"/>
-      <c r="E23" s="102">
+      <c r="B23" s="99" t="s">
+        <v>193</v>
+      </c>
+      <c r="C23" s="100"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="101">
         <v>4</v>
       </c>
-      <c r="F23" s="102"/>
-      <c r="G23" s="102"/>
-      <c r="H23" s="102">
+      <c r="F23" s="101"/>
+      <c r="G23" s="101"/>
+      <c r="H23" s="101">
         <f>SUM(E23:F23)</f>
         <v>4</v>
       </c>
-      <c r="I23" s="103">
+      <c r="I23" s="102">
         <f>E23*15+F23*30</f>
         <v>60</v>
       </c>
@@ -3094,24 +3096,24 @@
       <c r="Z23" s="26"/>
     </row>
     <row r="24" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="107" t="s">
+      <c r="A24" s="106" t="s">
         <v>108</v>
       </c>
-      <c r="B24" s="100" t="s">
+      <c r="B24" s="99" t="s">
         <v>109</v>
       </c>
-      <c r="C24" s="101"/>
-      <c r="D24" s="100"/>
-      <c r="E24" s="102">
+      <c r="C24" s="100"/>
+      <c r="D24" s="99"/>
+      <c r="E24" s="101">
         <v>3</v>
       </c>
-      <c r="F24" s="102"/>
-      <c r="G24" s="102"/>
-      <c r="H24" s="102">
+      <c r="F24" s="101"/>
+      <c r="G24" s="101"/>
+      <c r="H24" s="101">
         <f>SUM(E24:F24)</f>
         <v>3</v>
       </c>
-      <c r="I24" s="103">
+      <c r="I24" s="102">
         <f>E24*15+F24*30</f>
         <v>45</v>
       </c>
@@ -3134,24 +3136,24 @@
       <c r="Z24" s="26"/>
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="107" t="s">
+      <c r="A25" s="106" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="100" t="s">
+      <c r="B25" s="99" t="s">
         <v>111</v>
       </c>
-      <c r="C25" s="101"/>
-      <c r="D25" s="100"/>
-      <c r="E25" s="102">
+      <c r="C25" s="100"/>
+      <c r="D25" s="99"/>
+      <c r="E25" s="101">
         <v>3</v>
       </c>
-      <c r="F25" s="102"/>
-      <c r="G25" s="102"/>
-      <c r="H25" s="102">
+      <c r="F25" s="101"/>
+      <c r="G25" s="101"/>
+      <c r="H25" s="101">
         <f>SUM(E25:F25)</f>
         <v>3</v>
       </c>
-      <c r="I25" s="103">
+      <c r="I25" s="102">
         <f>E25*15+F25*30</f>
         <v>45</v>
       </c>
@@ -3174,12 +3176,12 @@
       <c r="Z25" s="26"/>
     </row>
     <row r="26" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="108"/>
-      <c r="B26" s="155" t="s">
+      <c r="A26" s="107"/>
+      <c r="B26" s="158" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="127"/>
-      <c r="D26" s="156"/>
+      <c r="C26" s="132"/>
+      <c r="D26" s="138"/>
       <c r="E26" s="40">
         <f>SUM(E21:E25)</f>
         <v>24</v>
@@ -3219,15 +3221,15 @@
       <c r="Z26" s="26"/>
     </row>
     <row r="27" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="135"/>
-      <c r="B27" s="126"/>
-      <c r="C27" s="127"/>
-      <c r="D27" s="126"/>
-      <c r="E27" s="127"/>
-      <c r="F27" s="127"/>
-      <c r="G27" s="127"/>
-      <c r="H27" s="127"/>
-      <c r="I27" s="128"/>
+      <c r="A27" s="130"/>
+      <c r="B27" s="131"/>
+      <c r="C27" s="132"/>
+      <c r="D27" s="131"/>
+      <c r="E27" s="132"/>
+      <c r="F27" s="132"/>
+      <c r="G27" s="132"/>
+      <c r="H27" s="132"/>
+      <c r="I27" s="133"/>
       <c r="J27" s="39"/>
       <c r="K27" s="26"/>
       <c r="L27" s="26"/>
@@ -3247,23 +3249,23 @@
       <c r="Z27" s="26"/>
     </row>
     <row r="28" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="134" t="s">
+      <c r="A28" s="159" t="s">
         <v>112</v>
       </c>
-      <c r="B28" s="156"/>
-      <c r="C28" s="178" t="s">
+      <c r="B28" s="138"/>
+      <c r="C28" s="139" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="180" t="s">
+      <c r="D28" s="141" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="182" t="s">
+      <c r="E28" s="143" t="s">
         <v>87</v>
       </c>
-      <c r="F28" s="127"/>
-      <c r="G28" s="127"/>
-      <c r="H28" s="183"/>
-      <c r="I28" s="184" t="s">
+      <c r="F28" s="132"/>
+      <c r="G28" s="132"/>
+      <c r="H28" s="136"/>
+      <c r="I28" s="144" t="s">
         <v>88</v>
       </c>
       <c r="J28" s="25"/>
@@ -3285,12 +3287,12 @@
       <c r="Z28" s="26"/>
     </row>
     <row r="29" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="134" t="s">
+      <c r="A29" s="159" t="s">
         <v>113</v>
       </c>
-      <c r="B29" s="156"/>
-      <c r="C29" s="179"/>
-      <c r="D29" s="181"/>
+      <c r="B29" s="138"/>
+      <c r="C29" s="140"/>
+      <c r="D29" s="142"/>
       <c r="E29" s="40" t="s">
         <v>90</v>
       </c>
@@ -3303,7 +3305,7 @@
       <c r="H29" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="I29" s="185"/>
+      <c r="I29" s="145"/>
       <c r="J29" s="25"/>
       <c r="K29" s="26"/>
       <c r="L29" s="26"/>
@@ -3323,17 +3325,17 @@
       <c r="Z29" s="26"/>
     </row>
     <row r="30" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="177" t="s">
+      <c r="A30" s="160" t="s">
         <v>114</v>
       </c>
-      <c r="B30" s="126"/>
-      <c r="C30" s="127"/>
-      <c r="D30" s="126"/>
-      <c r="E30" s="127"/>
-      <c r="F30" s="127"/>
-      <c r="G30" s="127"/>
-      <c r="H30" s="127"/>
-      <c r="I30" s="128"/>
+      <c r="B30" s="131"/>
+      <c r="C30" s="132"/>
+      <c r="D30" s="131"/>
+      <c r="E30" s="132"/>
+      <c r="F30" s="132"/>
+      <c r="G30" s="132"/>
+      <c r="H30" s="132"/>
+      <c r="I30" s="133"/>
       <c r="J30" s="25"/>
       <c r="K30" s="26"/>
       <c r="L30" s="26"/>
@@ -3353,14 +3355,14 @@
       <c r="Z30" s="26"/>
     </row>
     <row r="31" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="108" t="s">
+      <c r="A31" s="107" t="s">
         <v>115</v>
       </c>
       <c r="B31" s="41" t="s">
         <v>116</v>
       </c>
       <c r="C31" s="32" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D31" s="41"/>
       <c r="E31" s="42">
@@ -3397,14 +3399,14 @@
       <c r="Z31" s="26"/>
     </row>
     <row r="32" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="109" t="s">
-        <v>196</v>
-      </c>
-      <c r="B32" s="100" t="s">
+      <c r="A32" s="108" t="s">
+        <v>195</v>
+      </c>
+      <c r="B32" s="99" t="s">
         <v>117</v>
       </c>
-      <c r="C32" s="110" t="s">
-        <v>201</v>
+      <c r="C32" s="109" t="s">
+        <v>200</v>
       </c>
       <c r="D32" s="41"/>
       <c r="E32" s="42">
@@ -3439,17 +3441,17 @@
       <c r="Z32" s="26"/>
     </row>
     <row r="33" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="108" t="s">
+      <c r="A33" s="107" t="s">
         <v>118</v>
       </c>
-      <c r="B33" s="100" t="s">
-        <v>200</v>
-      </c>
-      <c r="C33" s="99" t="s">
-        <v>203</v>
+      <c r="B33" s="99" t="s">
+        <v>199</v>
+      </c>
+      <c r="C33" s="98" t="s">
+        <v>202</v>
       </c>
       <c r="D33" s="41"/>
-      <c r="E33" s="102">
+      <c r="E33" s="101">
         <v>4</v>
       </c>
       <c r="F33" s="42"/>
@@ -3481,14 +3483,14 @@
       <c r="Z33" s="26"/>
     </row>
     <row r="34" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="108" t="s">
+      <c r="A34" s="107" t="s">
         <v>119</v>
       </c>
-      <c r="B34" s="100" t="s">
-        <v>208</v>
-      </c>
-      <c r="C34" s="110" t="s">
-        <v>210</v>
+      <c r="B34" s="99" t="s">
+        <v>207</v>
+      </c>
+      <c r="C34" s="109" t="s">
+        <v>209</v>
       </c>
       <c r="D34" s="41"/>
       <c r="E34" s="42">
@@ -3523,14 +3525,14 @@
       <c r="Z34" s="26"/>
     </row>
     <row r="35" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="108" t="s">
+      <c r="A35" s="107" t="s">
         <v>120</v>
       </c>
-      <c r="B35" s="100" t="s">
+      <c r="B35" s="99" t="s">
         <v>121</v>
       </c>
-      <c r="C35" s="99" t="s">
-        <v>203</v>
+      <c r="C35" s="98" t="s">
+        <v>202</v>
       </c>
       <c r="D35" s="41"/>
       <c r="E35" s="42">
@@ -3566,11 +3568,11 @@
     </row>
     <row r="36" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="32"/>
-      <c r="B36" s="155" t="s">
+      <c r="B36" s="158" t="s">
         <v>102</v>
       </c>
-      <c r="C36" s="127"/>
-      <c r="D36" s="156"/>
+      <c r="C36" s="132"/>
+      <c r="D36" s="138"/>
       <c r="E36" s="40">
         <f>SUM(E31:E35)</f>
         <v>24</v>
@@ -3610,15 +3612,15 @@
       <c r="Z36" s="26"/>
     </row>
     <row r="37" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="135"/>
-      <c r="B37" s="126"/>
-      <c r="C37" s="127"/>
-      <c r="D37" s="126"/>
-      <c r="E37" s="127"/>
-      <c r="F37" s="127"/>
-      <c r="G37" s="127"/>
-      <c r="H37" s="127"/>
-      <c r="I37" s="128"/>
+      <c r="A37" s="130"/>
+      <c r="B37" s="131"/>
+      <c r="C37" s="132"/>
+      <c r="D37" s="131"/>
+      <c r="E37" s="132"/>
+      <c r="F37" s="132"/>
+      <c r="G37" s="132"/>
+      <c r="H37" s="132"/>
+      <c r="I37" s="133"/>
       <c r="J37" s="39"/>
       <c r="K37" s="26"/>
       <c r="L37" s="26"/>
@@ -3638,17 +3640,17 @@
       <c r="Z37" s="26"/>
     </row>
     <row r="38" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="125" t="s">
+      <c r="A38" s="161" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="126"/>
-      <c r="C38" s="127"/>
-      <c r="D38" s="126"/>
-      <c r="E38" s="127"/>
-      <c r="F38" s="127"/>
-      <c r="G38" s="127"/>
-      <c r="H38" s="127"/>
-      <c r="I38" s="128"/>
+      <c r="B38" s="131"/>
+      <c r="C38" s="132"/>
+      <c r="D38" s="131"/>
+      <c r="E38" s="132"/>
+      <c r="F38" s="132"/>
+      <c r="G38" s="132"/>
+      <c r="H38" s="132"/>
+      <c r="I38" s="133"/>
       <c r="J38" s="25"/>
       <c r="K38" s="26"/>
       <c r="L38" s="26"/>
@@ -3668,30 +3670,30 @@
       <c r="Z38" s="26"/>
     </row>
     <row r="39" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="107" t="s">
+      <c r="A39" s="106" t="s">
         <v>123</v>
       </c>
-      <c r="B39" s="100" t="s">
+      <c r="B39" s="99" t="s">
         <v>124</v>
       </c>
       <c r="C39" s="32" t="s">
-        <v>202</v>
-      </c>
-      <c r="D39" s="100"/>
-      <c r="E39" s="102">
+        <v>201</v>
+      </c>
+      <c r="D39" s="99"/>
+      <c r="E39" s="101">
         <v>4</v>
       </c>
-      <c r="F39" s="102">
+      <c r="F39" s="101">
         <v>4</v>
       </c>
-      <c r="G39" s="102">
+      <c r="G39" s="101">
         <v>4</v>
       </c>
-      <c r="H39" s="102">
+      <c r="H39" s="101">
         <f>SUM(E39:F39)</f>
         <v>8</v>
       </c>
-      <c r="I39" s="103">
+      <c r="I39" s="102">
         <f>E39*15+F39*30</f>
         <v>180</v>
       </c>
@@ -3714,26 +3716,26 @@
       <c r="Z39" s="26"/>
     </row>
     <row r="40" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="109" t="s">
-        <v>199</v>
-      </c>
-      <c r="B40" s="100" t="s">
+      <c r="A40" s="108" t="s">
+        <v>198</v>
+      </c>
+      <c r="B40" s="99" t="s">
         <v>125</v>
       </c>
-      <c r="C40" s="110" t="s">
-        <v>201</v>
-      </c>
-      <c r="D40" s="100"/>
-      <c r="E40" s="102">
+      <c r="C40" s="109" t="s">
+        <v>200</v>
+      </c>
+      <c r="D40" s="99"/>
+      <c r="E40" s="101">
         <v>11</v>
       </c>
-      <c r="F40" s="102"/>
-      <c r="G40" s="102"/>
-      <c r="H40" s="102">
+      <c r="F40" s="101"/>
+      <c r="G40" s="101"/>
+      <c r="H40" s="101">
         <f>SUM(E40:F40)</f>
         <v>11</v>
       </c>
-      <c r="I40" s="103">
+      <c r="I40" s="102">
         <f>E40*15+F40*30</f>
         <v>165</v>
       </c>
@@ -3756,26 +3758,26 @@
       <c r="Z40" s="26"/>
     </row>
     <row r="41" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="107" t="s">
+      <c r="A41" s="106" t="s">
         <v>126</v>
       </c>
-      <c r="B41" s="100" t="s">
+      <c r="B41" s="99" t="s">
         <v>127</v>
       </c>
-      <c r="C41" s="99" t="s">
-        <v>203</v>
-      </c>
-      <c r="D41" s="100"/>
-      <c r="E41" s="102">
+      <c r="C41" s="98" t="s">
+        <v>202</v>
+      </c>
+      <c r="D41" s="99"/>
+      <c r="E41" s="101">
         <v>3</v>
       </c>
-      <c r="F41" s="102"/>
-      <c r="G41" s="102"/>
-      <c r="H41" s="102">
+      <c r="F41" s="101"/>
+      <c r="G41" s="101"/>
+      <c r="H41" s="101">
         <f>SUM(E41:F41)</f>
         <v>3</v>
       </c>
-      <c r="I41" s="103">
+      <c r="I41" s="102">
         <f>E41*15+F41*30</f>
         <v>45</v>
       </c>
@@ -3798,26 +3800,26 @@
       <c r="Z41" s="26"/>
     </row>
     <row r="42" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="107" t="s">
+      <c r="A42" s="106" t="s">
         <v>128</v>
       </c>
-      <c r="B42" s="100" t="s">
+      <c r="B42" s="99" t="s">
         <v>129</v>
       </c>
-      <c r="C42" s="110" t="s">
-        <v>201</v>
-      </c>
-      <c r="D42" s="100"/>
-      <c r="E42" s="102">
+      <c r="C42" s="109" t="s">
+        <v>200</v>
+      </c>
+      <c r="D42" s="99"/>
+      <c r="E42" s="101">
         <v>3</v>
       </c>
-      <c r="F42" s="102"/>
-      <c r="G42" s="102"/>
-      <c r="H42" s="102">
+      <c r="F42" s="101"/>
+      <c r="G42" s="101"/>
+      <c r="H42" s="101">
         <f>SUM(E42:F42)</f>
         <v>3</v>
       </c>
-      <c r="I42" s="103">
+      <c r="I42" s="102">
         <f>E42*15+F42*30</f>
         <v>45</v>
       </c>
@@ -3840,26 +3842,26 @@
       <c r="Z42" s="26"/>
     </row>
     <row r="43" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="107" t="s">
+      <c r="A43" s="106" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="100" t="s">
+      <c r="B43" s="99" t="s">
         <v>131</v>
       </c>
-      <c r="C43" s="99" t="s">
-        <v>203</v>
-      </c>
-      <c r="D43" s="100"/>
-      <c r="E43" s="102">
+      <c r="C43" s="98" t="s">
+        <v>202</v>
+      </c>
+      <c r="D43" s="99"/>
+      <c r="E43" s="101">
         <v>4</v>
       </c>
-      <c r="F43" s="102"/>
-      <c r="G43" s="102"/>
-      <c r="H43" s="102">
+      <c r="F43" s="101"/>
+      <c r="G43" s="101"/>
+      <c r="H43" s="101">
         <f>SUM(E43:F43)</f>
         <v>4</v>
       </c>
-      <c r="I43" s="103">
+      <c r="I43" s="102">
         <f>E43*15+F43*30</f>
         <v>60</v>
       </c>
@@ -3882,29 +3884,29 @@
       <c r="Z43" s="26"/>
     </row>
     <row r="44" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="99"/>
-      <c r="B44" s="161" t="s">
+      <c r="A44" s="98"/>
+      <c r="B44" s="151" t="s">
         <v>102</v>
       </c>
-      <c r="C44" s="159"/>
-      <c r="D44" s="162"/>
-      <c r="E44" s="104">
+      <c r="C44" s="152"/>
+      <c r="D44" s="153"/>
+      <c r="E44" s="103">
         <f>SUM(E39:E43)</f>
         <v>25</v>
       </c>
-      <c r="F44" s="104">
+      <c r="F44" s="103">
         <f>SUM(F38:F43)</f>
         <v>4</v>
       </c>
-      <c r="G44" s="104">
+      <c r="G44" s="103">
         <f>SUM(G38:G43)</f>
         <v>4</v>
       </c>
-      <c r="H44" s="104">
+      <c r="H44" s="103">
         <f>SUM(H39:H43)</f>
         <v>29</v>
       </c>
-      <c r="I44" s="112">
+      <c r="I44" s="111">
         <f>SUM(I39:I43)</f>
         <v>495</v>
       </c>
@@ -3927,15 +3929,15 @@
       <c r="Z44" s="26"/>
     </row>
     <row r="45" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="164"/>
-      <c r="B45" s="165"/>
-      <c r="C45" s="166"/>
-      <c r="D45" s="165"/>
-      <c r="E45" s="166"/>
-      <c r="F45" s="166"/>
-      <c r="G45" s="166"/>
-      <c r="H45" s="166"/>
-      <c r="I45" s="167"/>
+      <c r="A45" s="162"/>
+      <c r="B45" s="163"/>
+      <c r="C45" s="164"/>
+      <c r="D45" s="163"/>
+      <c r="E45" s="164"/>
+      <c r="F45" s="164"/>
+      <c r="G45" s="164"/>
+      <c r="H45" s="164"/>
+      <c r="I45" s="165"/>
       <c r="J45" s="25"/>
       <c r="K45" s="26"/>
       <c r="L45" s="26"/>
@@ -3955,23 +3957,23 @@
       <c r="Z45" s="26"/>
     </row>
     <row r="46" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="168" t="s">
+      <c r="A46" s="166" t="s">
         <v>112</v>
       </c>
-      <c r="B46" s="162"/>
-      <c r="C46" s="169" t="s">
+      <c r="B46" s="153"/>
+      <c r="C46" s="167" t="s">
         <v>85</v>
       </c>
-      <c r="D46" s="171" t="s">
+      <c r="D46" s="169" t="s">
         <v>86</v>
       </c>
-      <c r="E46" s="173" t="s">
+      <c r="E46" s="171" t="s">
         <v>87</v>
       </c>
-      <c r="F46" s="159"/>
-      <c r="G46" s="159"/>
-      <c r="H46" s="174"/>
-      <c r="I46" s="175" t="s">
+      <c r="F46" s="152"/>
+      <c r="G46" s="152"/>
+      <c r="H46" s="172"/>
+      <c r="I46" s="173" t="s">
         <v>88</v>
       </c>
       <c r="J46" s="25"/>
@@ -3993,25 +3995,25 @@
       <c r="Z46" s="26"/>
     </row>
     <row r="47" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="168" t="s">
+      <c r="A47" s="166" t="s">
         <v>113</v>
       </c>
-      <c r="B47" s="162"/>
-      <c r="C47" s="170"/>
-      <c r="D47" s="172"/>
-      <c r="E47" s="104" t="s">
+      <c r="B47" s="153"/>
+      <c r="C47" s="168"/>
+      <c r="D47" s="170"/>
+      <c r="E47" s="103" t="s">
         <v>90</v>
       </c>
-      <c r="F47" s="104" t="s">
+      <c r="F47" s="103" t="s">
         <v>91</v>
       </c>
-      <c r="G47" s="104" t="s">
+      <c r="G47" s="103" t="s">
         <v>92</v>
       </c>
-      <c r="H47" s="104" t="s">
+      <c r="H47" s="103" t="s">
         <v>93</v>
       </c>
-      <c r="I47" s="176"/>
+      <c r="I47" s="174"/>
       <c r="J47" s="25"/>
       <c r="K47" s="26"/>
       <c r="L47" s="26"/>
@@ -4031,17 +4033,17 @@
       <c r="Z47" s="26"/>
     </row>
     <row r="48" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="157" t="s">
+      <c r="A48" s="175" t="s">
         <v>132</v>
       </c>
-      <c r="B48" s="158"/>
-      <c r="C48" s="159"/>
-      <c r="D48" s="158"/>
-      <c r="E48" s="159"/>
-      <c r="F48" s="159"/>
-      <c r="G48" s="159"/>
-      <c r="H48" s="159"/>
-      <c r="I48" s="160"/>
+      <c r="B48" s="155"/>
+      <c r="C48" s="152"/>
+      <c r="D48" s="155"/>
+      <c r="E48" s="152"/>
+      <c r="F48" s="152"/>
+      <c r="G48" s="152"/>
+      <c r="H48" s="152"/>
+      <c r="I48" s="156"/>
       <c r="J48" s="25"/>
       <c r="K48" s="26"/>
       <c r="L48" s="26"/>
@@ -4061,28 +4063,28 @@
       <c r="Z48" s="26"/>
     </row>
     <row r="49" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="107" t="s">
+      <c r="A49" s="106" t="s">
         <v>133</v>
       </c>
-      <c r="B49" s="100" t="s">
+      <c r="B49" s="99" t="s">
         <v>134</v>
       </c>
-      <c r="C49" s="99" t="s">
-        <v>204</v>
-      </c>
-      <c r="D49" s="100"/>
-      <c r="E49" s="102">
+      <c r="C49" s="98" t="s">
+        <v>203</v>
+      </c>
+      <c r="D49" s="99"/>
+      <c r="E49" s="101">
         <v>4</v>
       </c>
-      <c r="F49" s="102">
+      <c r="F49" s="101">
         <v>4</v>
       </c>
-      <c r="G49" s="102"/>
-      <c r="H49" s="102">
+      <c r="G49" s="101"/>
+      <c r="H49" s="101">
         <f>SUM(E49:F49)</f>
         <v>8</v>
       </c>
-      <c r="I49" s="103">
+      <c r="I49" s="102">
         <f>E49*15+F49*30</f>
         <v>180</v>
       </c>
@@ -4105,26 +4107,26 @@
       <c r="Z49" s="26"/>
     </row>
     <row r="50" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="109" t="s">
-        <v>198</v>
-      </c>
-      <c r="B50" s="100" t="s">
+      <c r="A50" s="108" t="s">
+        <v>197</v>
+      </c>
+      <c r="B50" s="99" t="s">
         <v>135</v>
       </c>
-      <c r="C50" s="110" t="s">
-        <v>205</v>
-      </c>
-      <c r="D50" s="100"/>
-      <c r="E50" s="102">
+      <c r="C50" s="109" t="s">
+        <v>204</v>
+      </c>
+      <c r="D50" s="99"/>
+      <c r="E50" s="101">
         <v>10</v>
       </c>
-      <c r="F50" s="102"/>
-      <c r="G50" s="102"/>
-      <c r="H50" s="102">
+      <c r="F50" s="101"/>
+      <c r="G50" s="101"/>
+      <c r="H50" s="101">
         <f>SUM(E50:F50)</f>
         <v>10</v>
       </c>
-      <c r="I50" s="103">
+      <c r="I50" s="102">
         <f>E50*15+F50*30</f>
         <v>150</v>
       </c>
@@ -4147,24 +4149,24 @@
       <c r="Z50" s="26"/>
     </row>
     <row r="51" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="107" t="s">
+      <c r="A51" s="106" t="s">
         <v>136</v>
       </c>
-      <c r="B51" s="100" t="s">
+      <c r="B51" s="99" t="s">
         <v>137</v>
       </c>
-      <c r="C51" s="111"/>
-      <c r="D51" s="100"/>
-      <c r="E51" s="102">
+      <c r="C51" s="110"/>
+      <c r="D51" s="99"/>
+      <c r="E51" s="101">
         <v>3</v>
       </c>
-      <c r="F51" s="102"/>
-      <c r="G51" s="102"/>
-      <c r="H51" s="102">
+      <c r="F51" s="101"/>
+      <c r="G51" s="101"/>
+      <c r="H51" s="101">
         <f>SUM(E51:F51)</f>
         <v>3</v>
       </c>
-      <c r="I51" s="103">
+      <c r="I51" s="102">
         <f>E51*15+F51*30</f>
         <v>45</v>
       </c>
@@ -4187,26 +4189,26 @@
       <c r="Z51" s="26"/>
     </row>
     <row r="52" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="107" t="s">
+      <c r="A52" s="106" t="s">
         <v>138</v>
       </c>
-      <c r="B52" s="100" t="s">
+      <c r="B52" s="99" t="s">
         <v>139</v>
       </c>
-      <c r="C52" s="99" t="s">
-        <v>211</v>
-      </c>
-      <c r="D52" s="100"/>
-      <c r="E52" s="102">
+      <c r="C52" s="98" t="s">
+        <v>210</v>
+      </c>
+      <c r="D52" s="99"/>
+      <c r="E52" s="101">
         <v>3</v>
       </c>
-      <c r="F52" s="102"/>
-      <c r="G52" s="102"/>
-      <c r="H52" s="102">
+      <c r="F52" s="101"/>
+      <c r="G52" s="101"/>
+      <c r="H52" s="101">
         <f>SUM(E52:F52)</f>
         <v>3</v>
       </c>
-      <c r="I52" s="103">
+      <c r="I52" s="102">
         <f>E52*15+F52*30</f>
         <v>45</v>
       </c>
@@ -4229,26 +4231,26 @@
       <c r="Z52" s="26"/>
     </row>
     <row r="53" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="107" t="s">
+      <c r="A53" s="106" t="s">
         <v>140</v>
       </c>
-      <c r="B53" s="100" t="s">
+      <c r="B53" s="99" t="s">
         <v>141</v>
       </c>
-      <c r="C53" s="99" t="s">
-        <v>211</v>
-      </c>
-      <c r="D53" s="100"/>
-      <c r="E53" s="102">
+      <c r="C53" s="98" t="s">
+        <v>210</v>
+      </c>
+      <c r="D53" s="99"/>
+      <c r="E53" s="101">
         <v>4</v>
       </c>
-      <c r="F53" s="102"/>
-      <c r="G53" s="102"/>
-      <c r="H53" s="102">
+      <c r="F53" s="101"/>
+      <c r="G53" s="101"/>
+      <c r="H53" s="101">
         <f>SUM(E53:F53)</f>
         <v>4</v>
       </c>
-      <c r="I53" s="103">
+      <c r="I53" s="102">
         <f>E53*15+F53*30</f>
         <v>60</v>
       </c>
@@ -4271,29 +4273,29 @@
       <c r="Z53" s="26"/>
     </row>
     <row r="54" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="99"/>
-      <c r="B54" s="161" t="s">
+      <c r="A54" s="98"/>
+      <c r="B54" s="151" t="s">
         <v>102</v>
       </c>
-      <c r="C54" s="159"/>
-      <c r="D54" s="162"/>
-      <c r="E54" s="104">
+      <c r="C54" s="152"/>
+      <c r="D54" s="153"/>
+      <c r="E54" s="103">
         <f>SUM(E49:E53)</f>
         <v>24</v>
       </c>
-      <c r="F54" s="104">
+      <c r="F54" s="103">
         <f>SUM(F49:F53)</f>
         <v>4</v>
       </c>
-      <c r="G54" s="104">
+      <c r="G54" s="103">
         <f>SUM(G49:G53)</f>
         <v>0</v>
       </c>
-      <c r="H54" s="104">
+      <c r="H54" s="103">
         <f>SUM(H49:H53)</f>
         <v>28</v>
       </c>
-      <c r="I54" s="112">
+      <c r="I54" s="111">
         <f>SUM(I49:I53)</f>
         <v>480</v>
       </c>
@@ -4316,15 +4318,15 @@
       <c r="Z54" s="26"/>
     </row>
     <row r="55" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="163"/>
-      <c r="B55" s="158"/>
-      <c r="C55" s="159"/>
-      <c r="D55" s="158"/>
-      <c r="E55" s="159"/>
-      <c r="F55" s="159"/>
-      <c r="G55" s="159"/>
-      <c r="H55" s="159"/>
-      <c r="I55" s="160"/>
+      <c r="A55" s="154"/>
+      <c r="B55" s="155"/>
+      <c r="C55" s="152"/>
+      <c r="D55" s="155"/>
+      <c r="E55" s="152"/>
+      <c r="F55" s="152"/>
+      <c r="G55" s="152"/>
+      <c r="H55" s="152"/>
+      <c r="I55" s="156"/>
       <c r="J55" s="25"/>
       <c r="K55" s="26"/>
       <c r="L55" s="26"/>
@@ -4344,17 +4346,17 @@
       <c r="Z55" s="26"/>
     </row>
     <row r="56" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="157" t="s">
+      <c r="A56" s="175" t="s">
         <v>142</v>
       </c>
-      <c r="B56" s="158"/>
-      <c r="C56" s="159"/>
-      <c r="D56" s="158"/>
-      <c r="E56" s="159"/>
-      <c r="F56" s="159"/>
-      <c r="G56" s="159"/>
-      <c r="H56" s="159"/>
-      <c r="I56" s="160"/>
+      <c r="B56" s="155"/>
+      <c r="C56" s="152"/>
+      <c r="D56" s="155"/>
+      <c r="E56" s="152"/>
+      <c r="F56" s="152"/>
+      <c r="G56" s="152"/>
+      <c r="H56" s="152"/>
+      <c r="I56" s="156"/>
       <c r="J56" s="25"/>
       <c r="K56" s="26"/>
       <c r="L56" s="26"/>
@@ -4374,28 +4376,28 @@
       <c r="Z56" s="26"/>
     </row>
     <row r="57" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="107" t="s">
+      <c r="A57" s="106" t="s">
         <v>143</v>
       </c>
-      <c r="B57" s="100" t="s">
+      <c r="B57" s="99" t="s">
         <v>144</v>
       </c>
-      <c r="C57" s="111"/>
-      <c r="D57" s="100"/>
-      <c r="E57" s="102">
+      <c r="C57" s="110"/>
+      <c r="D57" s="99"/>
+      <c r="E57" s="101">
         <v>4</v>
       </c>
-      <c r="F57" s="102">
+      <c r="F57" s="101">
         <v>4</v>
       </c>
-      <c r="G57" s="102">
+      <c r="G57" s="101">
         <v>4</v>
       </c>
-      <c r="H57" s="102">
+      <c r="H57" s="101">
         <f>SUM(E57:F57)</f>
         <v>8</v>
       </c>
-      <c r="I57" s="103">
+      <c r="I57" s="102">
         <f>E57*15+F57*30</f>
         <v>180</v>
       </c>
@@ -4418,26 +4420,26 @@
       <c r="Z57" s="26"/>
     </row>
     <row r="58" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="109" t="s">
-        <v>197</v>
-      </c>
-      <c r="B58" s="100" t="s">
+      <c r="A58" s="108" t="s">
+        <v>196</v>
+      </c>
+      <c r="B58" s="99" t="s">
         <v>145</v>
       </c>
-      <c r="C58" s="110" t="s">
-        <v>205</v>
-      </c>
-      <c r="D58" s="100"/>
-      <c r="E58" s="102">
+      <c r="C58" s="109" t="s">
+        <v>204</v>
+      </c>
+      <c r="D58" s="99"/>
+      <c r="E58" s="101">
         <v>10</v>
       </c>
-      <c r="F58" s="102"/>
-      <c r="G58" s="102"/>
-      <c r="H58" s="102">
+      <c r="F58" s="101"/>
+      <c r="G58" s="101"/>
+      <c r="H58" s="101">
         <f>SUM(E58:F58)</f>
         <v>10</v>
       </c>
-      <c r="I58" s="103">
+      <c r="I58" s="102">
         <f>E58*15+F58*30</f>
         <v>150</v>
       </c>
@@ -4460,26 +4462,26 @@
       <c r="Z58" s="26"/>
     </row>
     <row r="59" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="107" t="s">
+      <c r="A59" s="106" t="s">
         <v>146</v>
       </c>
-      <c r="B59" s="100" t="s">
-        <v>207</v>
-      </c>
-      <c r="C59" s="99" t="s">
-        <v>212</v>
-      </c>
-      <c r="D59" s="100"/>
-      <c r="E59" s="102">
+      <c r="B59" s="99" t="s">
+        <v>206</v>
+      </c>
+      <c r="C59" s="98" t="s">
+        <v>211</v>
+      </c>
+      <c r="D59" s="99"/>
+      <c r="E59" s="101">
         <v>3</v>
       </c>
-      <c r="F59" s="102"/>
-      <c r="G59" s="102"/>
-      <c r="H59" s="102">
+      <c r="F59" s="101"/>
+      <c r="G59" s="101"/>
+      <c r="H59" s="101">
         <f>SUM(E59:F59)</f>
         <v>3</v>
       </c>
-      <c r="I59" s="103">
+      <c r="I59" s="102">
         <f>E59*15+F59*30</f>
         <v>45</v>
       </c>
@@ -4502,26 +4504,26 @@
       <c r="Z59" s="26"/>
     </row>
     <row r="60" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="107" t="s">
+      <c r="A60" s="106" t="s">
         <v>147</v>
       </c>
-      <c r="B60" s="100" t="s">
-        <v>52</v>
-      </c>
-      <c r="C60" s="99" t="s">
+      <c r="B60" s="99" t="s">
         <v>213</v>
       </c>
-      <c r="D60" s="100"/>
-      <c r="E60" s="102">
+      <c r="C60" s="98" t="s">
+        <v>212</v>
+      </c>
+      <c r="D60" s="99"/>
+      <c r="E60" s="101">
         <v>3</v>
       </c>
-      <c r="F60" s="102"/>
-      <c r="G60" s="102"/>
-      <c r="H60" s="102">
+      <c r="F60" s="101"/>
+      <c r="G60" s="101"/>
+      <c r="H60" s="101">
         <f>SUM(E60:F60)</f>
         <v>3</v>
       </c>
-      <c r="I60" s="103">
+      <c r="I60" s="102">
         <f>E60*15+F60*30</f>
         <v>45</v>
       </c>
@@ -4544,24 +4546,24 @@
       <c r="Z60" s="26"/>
     </row>
     <row r="61" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="107" t="s">
+      <c r="A61" s="106" t="s">
         <v>148</v>
       </c>
-      <c r="B61" s="100" t="s">
+      <c r="B61" s="99" t="s">
         <v>149</v>
       </c>
-      <c r="C61" s="107"/>
-      <c r="D61" s="100"/>
-      <c r="E61" s="102">
+      <c r="C61" s="106"/>
+      <c r="D61" s="99"/>
+      <c r="E61" s="101">
         <v>3</v>
       </c>
-      <c r="F61" s="102"/>
-      <c r="G61" s="102"/>
-      <c r="H61" s="102">
+      <c r="F61" s="101"/>
+      <c r="G61" s="101"/>
+      <c r="H61" s="101">
         <f>SUM(E61:F61)</f>
         <v>3</v>
       </c>
-      <c r="I61" s="103">
+      <c r="I61" s="102">
         <f>E61*15+F61*30</f>
         <v>45</v>
       </c>
@@ -4584,29 +4586,29 @@
       <c r="Z61" s="26"/>
     </row>
     <row r="62" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="99"/>
-      <c r="B62" s="161" t="s">
+      <c r="A62" s="98"/>
+      <c r="B62" s="151" t="s">
         <v>102</v>
       </c>
-      <c r="C62" s="159"/>
-      <c r="D62" s="162"/>
-      <c r="E62" s="104">
+      <c r="C62" s="152"/>
+      <c r="D62" s="153"/>
+      <c r="E62" s="103">
         <f>SUM(E57:E61)</f>
         <v>23</v>
       </c>
-      <c r="F62" s="104">
+      <c r="F62" s="103">
         <f>SUM(F57:F61)</f>
         <v>4</v>
       </c>
-      <c r="G62" s="104">
+      <c r="G62" s="103">
         <f>SUM(G57:G61)</f>
         <v>4</v>
       </c>
-      <c r="H62" s="104">
+      <c r="H62" s="103">
         <f>SUM(H57:H61)</f>
         <v>27</v>
       </c>
-      <c r="I62" s="112">
+      <c r="I62" s="111">
         <f>SUM(I57:I61)</f>
         <v>465</v>
       </c>
@@ -4629,15 +4631,15 @@
       <c r="Z62" s="26"/>
     </row>
     <row r="63" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="113"/>
-      <c r="B63" s="114"/>
-      <c r="C63" s="115"/>
-      <c r="D63" s="114"/>
-      <c r="E63" s="116"/>
-      <c r="F63" s="116"/>
-      <c r="G63" s="116"/>
-      <c r="H63" s="116"/>
-      <c r="I63" s="117"/>
+      <c r="A63" s="112"/>
+      <c r="B63" s="113"/>
+      <c r="C63" s="114"/>
+      <c r="D63" s="113"/>
+      <c r="E63" s="115"/>
+      <c r="F63" s="115"/>
+      <c r="G63" s="115"/>
+      <c r="H63" s="115"/>
+      <c r="I63" s="116"/>
       <c r="J63" s="25"/>
       <c r="K63" s="26"/>
       <c r="L63" s="26"/>
@@ -4657,17 +4659,17 @@
       <c r="Z63" s="26"/>
     </row>
     <row r="64" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="157" t="s">
+      <c r="A64" s="175" t="s">
         <v>150</v>
       </c>
-      <c r="B64" s="158"/>
-      <c r="C64" s="159"/>
-      <c r="D64" s="158"/>
-      <c r="E64" s="159"/>
-      <c r="F64" s="159"/>
-      <c r="G64" s="159"/>
-      <c r="H64" s="159"/>
-      <c r="I64" s="160"/>
+      <c r="B64" s="155"/>
+      <c r="C64" s="152"/>
+      <c r="D64" s="155"/>
+      <c r="E64" s="152"/>
+      <c r="F64" s="152"/>
+      <c r="G64" s="152"/>
+      <c r="H64" s="152"/>
+      <c r="I64" s="156"/>
       <c r="J64" s="25"/>
       <c r="K64" s="26"/>
       <c r="L64" s="26"/>
@@ -4687,26 +4689,26 @@
       <c r="Z64" s="26"/>
     </row>
     <row r="65" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="107" t="s">
+      <c r="A65" s="106" t="s">
         <v>151</v>
       </c>
-      <c r="B65" s="100" t="s">
+      <c r="B65" s="99" t="s">
         <v>152</v>
       </c>
-      <c r="C65" s="99"/>
-      <c r="D65" s="100"/>
-      <c r="E65" s="102">
+      <c r="C65" s="98"/>
+      <c r="D65" s="99"/>
+      <c r="E65" s="101">
         <v>4</v>
       </c>
-      <c r="F65" s="102">
+      <c r="F65" s="101">
         <v>4</v>
       </c>
-      <c r="G65" s="102"/>
-      <c r="H65" s="102">
+      <c r="G65" s="101"/>
+      <c r="H65" s="101">
         <f>SUM(E65:F65)</f>
         <v>8</v>
       </c>
-      <c r="I65" s="103">
+      <c r="I65" s="102">
         <f>E65*15+F65*30</f>
         <v>180</v>
       </c>
@@ -4729,24 +4731,24 @@
       <c r="Z65" s="26"/>
     </row>
     <row r="66" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="106" t="s">
+      <c r="A66" s="105" t="s">
         <v>28</v>
       </c>
-      <c r="B66" s="118" t="s">
+      <c r="B66" s="117" t="s">
         <v>153</v>
       </c>
-      <c r="C66" s="99"/>
-      <c r="D66" s="100"/>
-      <c r="E66" s="102">
+      <c r="C66" s="98"/>
+      <c r="D66" s="99"/>
+      <c r="E66" s="101">
         <v>4</v>
       </c>
-      <c r="F66" s="102"/>
-      <c r="G66" s="102"/>
-      <c r="H66" s="102">
+      <c r="F66" s="101"/>
+      <c r="G66" s="101"/>
+      <c r="H66" s="101">
         <f>SUM(E66:F66)</f>
         <v>4</v>
       </c>
-      <c r="I66" s="103">
+      <c r="I66" s="102">
         <f>E66*15+F66*30</f>
         <v>60</v>
       </c>
@@ -4769,24 +4771,24 @@
       <c r="Z66" s="26"/>
     </row>
     <row r="67" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="106" t="s">
+      <c r="A67" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="B67" s="118" t="s">
+      <c r="B67" s="117" t="s">
         <v>9</v>
       </c>
-      <c r="C67" s="99"/>
-      <c r="D67" s="100"/>
-      <c r="E67" s="102">
+      <c r="C67" s="98"/>
+      <c r="D67" s="99"/>
+      <c r="E67" s="101">
         <v>4</v>
       </c>
-      <c r="F67" s="102"/>
-      <c r="G67" s="102"/>
-      <c r="H67" s="102">
+      <c r="F67" s="101"/>
+      <c r="G67" s="101"/>
+      <c r="H67" s="101">
         <f>SUM(E67:F67)</f>
         <v>4</v>
       </c>
-      <c r="I67" s="103">
+      <c r="I67" s="102">
         <f>E67*15+F67*30</f>
         <v>60</v>
       </c>
@@ -4809,24 +4811,24 @@
       <c r="Z67" s="26"/>
     </row>
     <row r="68" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="106" t="s">
+      <c r="A68" s="105" t="s">
         <v>154</v>
       </c>
-      <c r="B68" s="118" t="s">
+      <c r="B68" s="117" t="s">
         <v>155</v>
       </c>
-      <c r="C68" s="99"/>
-      <c r="D68" s="100"/>
-      <c r="E68" s="102">
+      <c r="C68" s="98"/>
+      <c r="D68" s="99"/>
+      <c r="E68" s="101">
         <v>4</v>
       </c>
-      <c r="F68" s="102"/>
-      <c r="G68" s="102"/>
-      <c r="H68" s="102">
+      <c r="F68" s="101"/>
+      <c r="G68" s="101"/>
+      <c r="H68" s="101">
         <f>SUM(E68:F68)</f>
         <v>4</v>
       </c>
-      <c r="I68" s="103">
+      <c r="I68" s="102">
         <f>E68*15+F68*30</f>
         <v>60</v>
       </c>
@@ -4849,24 +4851,24 @@
       <c r="Z68" s="26"/>
     </row>
     <row r="69" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="106" t="s">
+      <c r="A69" s="105" t="s">
         <v>156</v>
       </c>
-      <c r="B69" s="118" t="s">
+      <c r="B69" s="117" t="s">
         <v>157</v>
       </c>
-      <c r="C69" s="99"/>
-      <c r="D69" s="100"/>
-      <c r="E69" s="102">
+      <c r="C69" s="98"/>
+      <c r="D69" s="99"/>
+      <c r="E69" s="101">
         <v>4</v>
       </c>
-      <c r="F69" s="102"/>
-      <c r="G69" s="102"/>
-      <c r="H69" s="102">
+      <c r="F69" s="101"/>
+      <c r="G69" s="101"/>
+      <c r="H69" s="101">
         <f>SUM(E69:F69)</f>
         <v>4</v>
       </c>
-      <c r="I69" s="103">
+      <c r="I69" s="102">
         <f>E69*15+F69*30</f>
         <v>60</v>
       </c>
@@ -4889,29 +4891,29 @@
       <c r="Z69" s="26"/>
     </row>
     <row r="70" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="99"/>
-      <c r="B70" s="161" t="s">
+      <c r="A70" s="98"/>
+      <c r="B70" s="151" t="s">
         <v>102</v>
       </c>
-      <c r="C70" s="159"/>
-      <c r="D70" s="162"/>
-      <c r="E70" s="104">
+      <c r="C70" s="152"/>
+      <c r="D70" s="153"/>
+      <c r="E70" s="103">
         <f>SUM(E65:E69)</f>
         <v>20</v>
       </c>
-      <c r="F70" s="104">
+      <c r="F70" s="103">
         <f>SUM(F65:F69)</f>
         <v>4</v>
       </c>
-      <c r="G70" s="104">
+      <c r="G70" s="103">
         <f>SUM(G65:G69)</f>
         <v>0</v>
       </c>
-      <c r="H70" s="104">
+      <c r="H70" s="103">
         <f>SUM(H65:H69)</f>
         <v>24</v>
       </c>
-      <c r="I70" s="112">
+      <c r="I70" s="111">
         <f>SUM(I65:I69)</f>
         <v>420</v>
       </c>
@@ -4934,15 +4936,15 @@
       <c r="Z70" s="26"/>
     </row>
     <row r="71" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="113"/>
-      <c r="B71" s="114"/>
-      <c r="C71" s="115"/>
-      <c r="D71" s="114"/>
-      <c r="E71" s="116"/>
-      <c r="F71" s="116"/>
-      <c r="G71" s="116"/>
-      <c r="H71" s="116"/>
-      <c r="I71" s="117"/>
+      <c r="A71" s="112"/>
+      <c r="B71" s="113"/>
+      <c r="C71" s="114"/>
+      <c r="D71" s="113"/>
+      <c r="E71" s="115"/>
+      <c r="F71" s="115"/>
+      <c r="G71" s="115"/>
+      <c r="H71" s="115"/>
+      <c r="I71" s="116"/>
       <c r="J71" s="25"/>
       <c r="K71" s="26"/>
       <c r="L71" s="26"/>
@@ -4962,17 +4964,17 @@
       <c r="Z71" s="26"/>
     </row>
     <row r="72" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="157" t="s">
+      <c r="A72" s="175" t="s">
         <v>158</v>
       </c>
-      <c r="B72" s="158"/>
-      <c r="C72" s="159"/>
-      <c r="D72" s="158"/>
-      <c r="E72" s="159"/>
-      <c r="F72" s="159"/>
-      <c r="G72" s="159"/>
-      <c r="H72" s="159"/>
-      <c r="I72" s="160"/>
+      <c r="B72" s="155"/>
+      <c r="C72" s="152"/>
+      <c r="D72" s="155"/>
+      <c r="E72" s="152"/>
+      <c r="F72" s="152"/>
+      <c r="G72" s="152"/>
+      <c r="H72" s="152"/>
+      <c r="I72" s="156"/>
       <c r="J72" s="25"/>
       <c r="K72" s="26"/>
       <c r="L72" s="26"/>
@@ -4992,28 +4994,28 @@
       <c r="Z72" s="26"/>
     </row>
     <row r="73" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="99" t="s">
+      <c r="A73" s="98" t="s">
         <v>159</v>
       </c>
-      <c r="B73" s="100" t="s">
+      <c r="B73" s="99" t="s">
         <v>160</v>
       </c>
-      <c r="C73" s="111"/>
-      <c r="D73" s="100"/>
-      <c r="E73" s="102">
+      <c r="C73" s="110"/>
+      <c r="D73" s="99"/>
+      <c r="E73" s="101">
         <v>4</v>
       </c>
-      <c r="F73" s="102">
+      <c r="F73" s="101">
         <v>4</v>
       </c>
-      <c r="G73" s="102">
+      <c r="G73" s="101">
         <v>4</v>
       </c>
-      <c r="H73" s="102">
+      <c r="H73" s="101">
         <f t="shared" ref="H73:H78" si="0">SUM(E73:F73)</f>
         <v>8</v>
       </c>
-      <c r="I73" s="103">
+      <c r="I73" s="102">
         <f t="shared" ref="I73:I78" si="1">E73*15+F73*30</f>
         <v>180</v>
       </c>
@@ -5036,24 +5038,24 @@
       <c r="Z73" s="26"/>
     </row>
     <row r="74" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="99" t="s">
+      <c r="A74" s="98" t="s">
         <v>161</v>
       </c>
-      <c r="B74" s="118" t="s">
+      <c r="B74" s="117" t="s">
         <v>162</v>
       </c>
-      <c r="C74" s="111"/>
-      <c r="D74" s="100"/>
-      <c r="E74" s="102">
+      <c r="C74" s="110"/>
+      <c r="D74" s="99"/>
+      <c r="E74" s="101">
         <v>2</v>
       </c>
-      <c r="F74" s="102"/>
-      <c r="G74" s="102"/>
-      <c r="H74" s="102">
+      <c r="F74" s="101"/>
+      <c r="G74" s="101"/>
+      <c r="H74" s="101">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I74" s="103">
+      <c r="I74" s="102">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
@@ -5076,24 +5078,24 @@
       <c r="Z74" s="26"/>
     </row>
     <row r="75" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="99" t="s">
-        <v>209</v>
-      </c>
-      <c r="B75" s="118" t="s">
+      <c r="A75" s="98" t="s">
+        <v>208</v>
+      </c>
+      <c r="B75" s="117" t="s">
         <v>163</v>
       </c>
-      <c r="C75" s="111"/>
-      <c r="D75" s="100"/>
-      <c r="E75" s="102">
+      <c r="C75" s="110"/>
+      <c r="D75" s="99"/>
+      <c r="E75" s="101">
         <v>2</v>
       </c>
-      <c r="F75" s="102"/>
-      <c r="G75" s="102"/>
-      <c r="H75" s="102">
+      <c r="F75" s="101"/>
+      <c r="G75" s="101"/>
+      <c r="H75" s="101">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I75" s="103">
+      <c r="I75" s="102">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
@@ -5116,22 +5118,22 @@
       <c r="Z75" s="26"/>
     </row>
     <row r="76" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="99" t="s">
+      <c r="A76" s="98" t="s">
         <v>164</v>
       </c>
-      <c r="B76" s="118"/>
-      <c r="C76" s="111"/>
-      <c r="D76" s="100"/>
-      <c r="E76" s="102">
+      <c r="B76" s="117"/>
+      <c r="C76" s="110"/>
+      <c r="D76" s="99"/>
+      <c r="E76" s="101">
         <v>4</v>
       </c>
-      <c r="F76" s="102"/>
-      <c r="G76" s="102"/>
-      <c r="H76" s="102">
+      <c r="F76" s="101"/>
+      <c r="G76" s="101"/>
+      <c r="H76" s="101">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I76" s="103">
+      <c r="I76" s="102">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
@@ -5154,22 +5156,22 @@
       <c r="Z76" s="26"/>
     </row>
     <row r="77" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="99" t="s">
+      <c r="A77" s="98" t="s">
         <v>164</v>
       </c>
-      <c r="B77" s="118"/>
-      <c r="C77" s="111"/>
-      <c r="D77" s="100"/>
-      <c r="E77" s="102">
+      <c r="B77" s="117"/>
+      <c r="C77" s="110"/>
+      <c r="D77" s="99"/>
+      <c r="E77" s="101">
         <v>4</v>
       </c>
-      <c r="F77" s="102"/>
-      <c r="G77" s="102"/>
-      <c r="H77" s="102">
+      <c r="F77" s="101"/>
+      <c r="G77" s="101"/>
+      <c r="H77" s="101">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I77" s="103">
+      <c r="I77" s="102">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
@@ -5192,22 +5194,22 @@
       <c r="Z77" s="26"/>
     </row>
     <row r="78" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="99" t="s">
+      <c r="A78" s="98" t="s">
         <v>164</v>
       </c>
-      <c r="B78" s="118"/>
-      <c r="C78" s="111"/>
-      <c r="D78" s="100"/>
-      <c r="E78" s="102">
+      <c r="B78" s="117"/>
+      <c r="C78" s="110"/>
+      <c r="D78" s="99"/>
+      <c r="E78" s="101">
         <v>4</v>
       </c>
-      <c r="F78" s="102"/>
-      <c r="G78" s="102"/>
-      <c r="H78" s="102">
+      <c r="F78" s="101"/>
+      <c r="G78" s="101"/>
+      <c r="H78" s="101">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I78" s="103">
+      <c r="I78" s="102">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
@@ -5230,29 +5232,29 @@
       <c r="Z78" s="26"/>
     </row>
     <row r="79" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="99"/>
-      <c r="B79" s="161" t="s">
+      <c r="A79" s="98"/>
+      <c r="B79" s="151" t="s">
         <v>102</v>
       </c>
-      <c r="C79" s="159"/>
-      <c r="D79" s="162"/>
-      <c r="E79" s="104">
+      <c r="C79" s="152"/>
+      <c r="D79" s="153"/>
+      <c r="E79" s="103">
         <f>SUM(E73:E78)</f>
         <v>20</v>
       </c>
-      <c r="F79" s="104">
+      <c r="F79" s="103">
         <f>SUM(F73:F78)</f>
         <v>4</v>
       </c>
-      <c r="G79" s="104">
+      <c r="G79" s="103">
         <f>SUM(G73:G78)</f>
         <v>4</v>
       </c>
-      <c r="H79" s="104">
+      <c r="H79" s="103">
         <f>SUM(H73:H78)</f>
         <v>24</v>
       </c>
-      <c r="I79" s="112">
+      <c r="I79" s="111">
         <f>SUM(I73:I78)</f>
         <v>420</v>
       </c>
@@ -5275,15 +5277,15 @@
       <c r="Z79" s="26"/>
     </row>
     <row r="80" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="113"/>
-      <c r="B80" s="114"/>
-      <c r="C80" s="115"/>
-      <c r="D80" s="114"/>
-      <c r="E80" s="116"/>
-      <c r="F80" s="116"/>
-      <c r="G80" s="116"/>
-      <c r="H80" s="116"/>
-      <c r="I80" s="117"/>
+      <c r="A80" s="112"/>
+      <c r="B80" s="113"/>
+      <c r="C80" s="114"/>
+      <c r="D80" s="113"/>
+      <c r="E80" s="115"/>
+      <c r="F80" s="115"/>
+      <c r="G80" s="115"/>
+      <c r="H80" s="115"/>
+      <c r="I80" s="116"/>
       <c r="J80" s="25"/>
       <c r="K80" s="26"/>
       <c r="L80" s="26"/>
@@ -5303,17 +5305,17 @@
       <c r="Z80" s="26"/>
     </row>
     <row r="81" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="157" t="s">
+      <c r="A81" s="175" t="s">
         <v>165</v>
       </c>
-      <c r="B81" s="158"/>
-      <c r="C81" s="159"/>
-      <c r="D81" s="158"/>
-      <c r="E81" s="159"/>
-      <c r="F81" s="159"/>
-      <c r="G81" s="159"/>
-      <c r="H81" s="159"/>
-      <c r="I81" s="160"/>
+      <c r="B81" s="155"/>
+      <c r="C81" s="152"/>
+      <c r="D81" s="155"/>
+      <c r="E81" s="152"/>
+      <c r="F81" s="152"/>
+      <c r="G81" s="152"/>
+      <c r="H81" s="152"/>
+      <c r="I81" s="156"/>
       <c r="J81" s="25"/>
       <c r="K81" s="26"/>
       <c r="L81" s="26"/>
@@ -5333,28 +5335,28 @@
       <c r="Z81" s="26"/>
     </row>
     <row r="82" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="99" t="s">
+      <c r="A82" s="98" t="s">
         <v>166</v>
       </c>
-      <c r="B82" s="118" t="s">
+      <c r="B82" s="117" t="s">
         <v>167</v>
       </c>
-      <c r="C82" s="99" t="s">
+      <c r="C82" s="98" t="s">
         <v>159</v>
       </c>
-      <c r="D82" s="119"/>
-      <c r="E82" s="120">
+      <c r="D82" s="118"/>
+      <c r="E82" s="119">
         <v>2</v>
       </c>
-      <c r="F82" s="120">
+      <c r="F82" s="119">
         <v>2</v>
       </c>
-      <c r="G82" s="102"/>
-      <c r="H82" s="102">
+      <c r="G82" s="101"/>
+      <c r="H82" s="101">
         <f>SUM(E82:F82)</f>
         <v>4</v>
       </c>
-      <c r="I82" s="103">
+      <c r="I82" s="102">
         <f>E82*15+F82*30</f>
         <v>90</v>
       </c>
@@ -5377,24 +5379,24 @@
       <c r="Z82" s="26"/>
     </row>
     <row r="83" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="99" t="s">
+      <c r="A83" s="98" t="s">
         <v>164</v>
       </c>
-      <c r="B83" s="118"/>
-      <c r="C83" s="121"/>
-      <c r="D83" s="118"/>
-      <c r="E83" s="120">
+      <c r="B83" s="117"/>
+      <c r="C83" s="120"/>
+      <c r="D83" s="117"/>
+      <c r="E83" s="119">
         <v>4</v>
       </c>
-      <c r="F83" s="120">
+      <c r="F83" s="119">
         <v>0</v>
       </c>
-      <c r="G83" s="102"/>
-      <c r="H83" s="102">
+      <c r="G83" s="101"/>
+      <c r="H83" s="101">
         <f>SUM(E83:F83)</f>
         <v>4</v>
       </c>
-      <c r="I83" s="103">
+      <c r="I83" s="102">
         <f>E83*15+F83*30</f>
         <v>60</v>
       </c>
@@ -5417,24 +5419,24 @@
       <c r="Z83" s="26"/>
     </row>
     <row r="84" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="99" t="s">
+      <c r="A84" s="98" t="s">
         <v>164</v>
       </c>
-      <c r="B84" s="118"/>
-      <c r="C84" s="111"/>
-      <c r="D84" s="118"/>
-      <c r="E84" s="120">
+      <c r="B84" s="117"/>
+      <c r="C84" s="110"/>
+      <c r="D84" s="117"/>
+      <c r="E84" s="119">
         <v>4</v>
       </c>
-      <c r="F84" s="120">
+      <c r="F84" s="119">
         <v>0</v>
       </c>
-      <c r="G84" s="102"/>
-      <c r="H84" s="102">
+      <c r="G84" s="101"/>
+      <c r="H84" s="101">
         <f>SUM(E84:F84)</f>
         <v>4</v>
       </c>
-      <c r="I84" s="103">
+      <c r="I84" s="102">
         <f>E84*15+F84*30</f>
         <v>60</v>
       </c>
@@ -5457,24 +5459,24 @@
       <c r="Z84" s="26"/>
     </row>
     <row r="85" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="99" t="s">
+      <c r="A85" s="98" t="s">
         <v>164</v>
       </c>
-      <c r="B85" s="122"/>
-      <c r="C85" s="123"/>
-      <c r="D85" s="122"/>
-      <c r="E85" s="124">
+      <c r="B85" s="121"/>
+      <c r="C85" s="122"/>
+      <c r="D85" s="121"/>
+      <c r="E85" s="123">
         <v>4</v>
       </c>
-      <c r="F85" s="124">
+      <c r="F85" s="123">
         <v>0</v>
       </c>
-      <c r="G85" s="102"/>
-      <c r="H85" s="102">
+      <c r="G85" s="101"/>
+      <c r="H85" s="101">
         <f>SUM(E85:F85)</f>
         <v>4</v>
       </c>
-      <c r="I85" s="103">
+      <c r="I85" s="102">
         <f>E85*15+F85*30</f>
         <v>60</v>
       </c>
@@ -5498,11 +5500,11 @@
     </row>
     <row r="86" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="32"/>
-      <c r="B86" s="155" t="s">
+      <c r="B86" s="158" t="s">
         <v>102</v>
       </c>
-      <c r="C86" s="127"/>
-      <c r="D86" s="156"/>
+      <c r="C86" s="132"/>
+      <c r="D86" s="138"/>
       <c r="E86" s="40">
         <f>SUM(E82:E85)</f>
         <v>14</v>
@@ -5570,17 +5572,17 @@
       <c r="Z87" s="26"/>
     </row>
     <row r="88" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="125" t="s">
+      <c r="A88" s="161" t="s">
         <v>168</v>
       </c>
-      <c r="B88" s="126"/>
-      <c r="C88" s="127"/>
-      <c r="D88" s="126"/>
-      <c r="E88" s="127"/>
-      <c r="F88" s="127"/>
-      <c r="G88" s="127"/>
-      <c r="H88" s="127"/>
-      <c r="I88" s="128"/>
+      <c r="B88" s="131"/>
+      <c r="C88" s="132"/>
+      <c r="D88" s="131"/>
+      <c r="E88" s="132"/>
+      <c r="F88" s="132"/>
+      <c r="G88" s="132"/>
+      <c r="H88" s="132"/>
+      <c r="I88" s="133"/>
       <c r="J88" s="25"/>
       <c r="K88" s="26"/>
       <c r="L88" s="26"/>
@@ -5805,11 +5807,11 @@
     </row>
     <row r="94" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="32"/>
-      <c r="B94" s="155" t="s">
+      <c r="B94" s="158" t="s">
         <v>102</v>
       </c>
-      <c r="C94" s="127"/>
-      <c r="D94" s="156"/>
+      <c r="C94" s="132"/>
+      <c r="D94" s="138"/>
       <c r="E94" s="40">
         <f>SUM(E89:E93)</f>
         <v>15</v>
@@ -5849,15 +5851,15 @@
       <c r="Z94" s="26"/>
     </row>
     <row r="95" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="133"/>
-      <c r="B95" s="126"/>
-      <c r="C95" s="127"/>
-      <c r="D95" s="126"/>
-      <c r="E95" s="127"/>
-      <c r="F95" s="127"/>
-      <c r="G95" s="127"/>
-      <c r="H95" s="127"/>
-      <c r="I95" s="128"/>
+      <c r="A95" s="134"/>
+      <c r="B95" s="131"/>
+      <c r="C95" s="132"/>
+      <c r="D95" s="131"/>
+      <c r="E95" s="132"/>
+      <c r="F95" s="132"/>
+      <c r="G95" s="132"/>
+      <c r="H95" s="132"/>
+      <c r="I95" s="133"/>
       <c r="J95" s="25"/>
       <c r="K95" s="26"/>
       <c r="L95" s="26"/>
@@ -5877,15 +5879,15 @@
       <c r="Z95" s="26"/>
     </row>
     <row r="96" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="133"/>
-      <c r="B96" s="126"/>
-      <c r="C96" s="127"/>
-      <c r="D96" s="126"/>
-      <c r="E96" s="127"/>
-      <c r="F96" s="127"/>
-      <c r="G96" s="127"/>
-      <c r="H96" s="127"/>
-      <c r="I96" s="128"/>
+      <c r="A96" s="134"/>
+      <c r="B96" s="131"/>
+      <c r="C96" s="132"/>
+      <c r="D96" s="131"/>
+      <c r="E96" s="132"/>
+      <c r="F96" s="132"/>
+      <c r="G96" s="132"/>
+      <c r="H96" s="132"/>
+      <c r="I96" s="133"/>
       <c r="J96" s="25"/>
       <c r="K96" s="26"/>
       <c r="L96" s="26"/>
@@ -5905,17 +5907,17 @@
       <c r="Z96" s="26"/>
     </row>
     <row r="97" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="135" t="s">
+      <c r="A97" s="130" t="s">
         <v>173</v>
       </c>
-      <c r="B97" s="126"/>
-      <c r="C97" s="127"/>
-      <c r="D97" s="126"/>
-      <c r="E97" s="127"/>
-      <c r="F97" s="127"/>
-      <c r="G97" s="127"/>
-      <c r="H97" s="127"/>
-      <c r="I97" s="128"/>
+      <c r="B97" s="131"/>
+      <c r="C97" s="132"/>
+      <c r="D97" s="131"/>
+      <c r="E97" s="132"/>
+      <c r="F97" s="132"/>
+      <c r="G97" s="132"/>
+      <c r="H97" s="132"/>
+      <c r="I97" s="133"/>
       <c r="J97" s="25"/>
       <c r="K97" s="26"/>
       <c r="L97" s="26"/>
@@ -5935,17 +5937,17 @@
       <c r="Z97" s="26"/>
     </row>
     <row r="98" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="135" t="s">
+      <c r="A98" s="130" t="s">
         <v>174</v>
       </c>
-      <c r="B98" s="126"/>
-      <c r="C98" s="127"/>
-      <c r="D98" s="126"/>
-      <c r="E98" s="127"/>
-      <c r="F98" s="127"/>
-      <c r="G98" s="127"/>
-      <c r="H98" s="127"/>
-      <c r="I98" s="128"/>
+      <c r="B98" s="131"/>
+      <c r="C98" s="132"/>
+      <c r="D98" s="131"/>
+      <c r="E98" s="132"/>
+      <c r="F98" s="132"/>
+      <c r="G98" s="132"/>
+      <c r="H98" s="132"/>
+      <c r="I98" s="133"/>
       <c r="J98" s="25"/>
       <c r="K98" s="26"/>
       <c r="L98" s="26"/>
@@ -5965,15 +5967,15 @@
       <c r="Z98" s="26"/>
     </row>
     <row r="99" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="133"/>
-      <c r="B99" s="126"/>
-      <c r="C99" s="127"/>
-      <c r="D99" s="126"/>
-      <c r="E99" s="127"/>
-      <c r="F99" s="131"/>
-      <c r="G99" s="131"/>
-      <c r="H99" s="131"/>
-      <c r="I99" s="128"/>
+      <c r="A99" s="134"/>
+      <c r="B99" s="131"/>
+      <c r="C99" s="132"/>
+      <c r="D99" s="131"/>
+      <c r="E99" s="132"/>
+      <c r="F99" s="149"/>
+      <c r="G99" s="149"/>
+      <c r="H99" s="149"/>
+      <c r="I99" s="133"/>
       <c r="J99" s="25"/>
       <c r="K99" s="26"/>
       <c r="L99" s="26"/>
@@ -5997,26 +5999,26 @@
       <c r="B100" s="60" t="s">
         <v>175</v>
       </c>
-      <c r="C100" s="154" t="s">
+      <c r="C100" s="176" t="s">
         <v>176</v>
       </c>
-      <c r="D100" s="130"/>
+      <c r="D100" s="148"/>
       <c r="E100" s="61">
         <f>SUM(E18+E26+E36+E44+E54+E62+E70+E79+E86+E94)</f>
         <v>213</v>
       </c>
-      <c r="F100" s="150" t="str">
+      <c r="F100" s="177" t="str">
         <f>E100*15&amp;" horas"</f>
         <v>3195 horas</v>
       </c>
-      <c r="G100" s="151"/>
-      <c r="H100" s="151"/>
+      <c r="G100" s="178"/>
+      <c r="H100" s="178"/>
       <c r="I100" s="62"/>
       <c r="J100" s="25"/>
-      <c r="K100" s="147" t="s">
+      <c r="K100" s="179" t="s">
         <v>176</v>
       </c>
-      <c r="L100" s="130"/>
+      <c r="L100" s="148"/>
       <c r="M100" s="26" t="s">
         <v>177</v>
       </c>
@@ -6043,26 +6045,26 @@
     <row r="101" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="28"/>
       <c r="B101" s="65"/>
-      <c r="C101" s="148" t="s">
+      <c r="C101" s="180" t="s">
         <v>178</v>
       </c>
-      <c r="D101" s="149"/>
+      <c r="D101" s="181"/>
       <c r="E101" s="66">
         <f>SUM(F18+F26+F36+F44+F54+F62+F70+F79+F86+F94)</f>
         <v>42</v>
       </c>
-      <c r="F101" s="150" t="str">
+      <c r="F101" s="177" t="str">
         <f>E101*30&amp;" horas"</f>
         <v>1260 horas</v>
       </c>
-      <c r="G101" s="151"/>
-      <c r="H101" s="151"/>
+      <c r="G101" s="178"/>
+      <c r="H101" s="178"/>
       <c r="I101" s="62"/>
       <c r="J101" s="25"/>
-      <c r="K101" s="147" t="s">
+      <c r="K101" s="179" t="s">
         <v>176</v>
       </c>
-      <c r="L101" s="130"/>
+      <c r="L101" s="148"/>
       <c r="M101" s="26" t="s">
         <v>179</v>
       </c>
@@ -6089,20 +6091,20 @@
     <row r="102" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="28"/>
       <c r="B102" s="60"/>
-      <c r="C102" s="152" t="s">
+      <c r="C102" s="182" t="s">
         <v>180</v>
       </c>
-      <c r="D102" s="153"/>
+      <c r="D102" s="183"/>
       <c r="E102" s="67">
         <f>SUM(G94+G86+G79+G70+G62+G54+G44+G26+G36+G18)</f>
         <v>16</v>
       </c>
-      <c r="F102" s="150" t="str">
+      <c r="F102" s="177" t="str">
         <f>E102*30&amp;" horas"</f>
         <v>480 horas</v>
       </c>
-      <c r="G102" s="151"/>
-      <c r="H102" s="151"/>
+      <c r="G102" s="178"/>
+      <c r="H102" s="178"/>
       <c r="I102" s="62"/>
       <c r="J102" s="25"/>
       <c r="K102" s="26"/>
@@ -6124,21 +6126,21 @@
     </row>
     <row r="103" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="68"/>
-      <c r="B103" s="136" t="s">
+      <c r="B103" s="184" t="s">
         <v>181</v>
       </c>
-      <c r="C103" s="137"/>
-      <c r="D103" s="138"/>
+      <c r="C103" s="185"/>
+      <c r="D103" s="186"/>
       <c r="E103" s="69">
         <f>SUM(E100:E101)</f>
         <v>255</v>
       </c>
-      <c r="F103" s="139">
+      <c r="F103" s="187">
         <f>SUM(E100)*15+SUM(E101)*"30"</f>
         <v>4455</v>
       </c>
-      <c r="G103" s="140"/>
-      <c r="H103" s="141"/>
+      <c r="G103" s="188"/>
+      <c r="H103" s="189"/>
       <c r="I103" s="70"/>
       <c r="J103" s="25"/>
       <c r="K103" s="26"/>
@@ -6187,16 +6189,16 @@
       <c r="Z104" s="26"/>
     </row>
     <row r="105" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="142" t="s">
+      <c r="A105" s="190" t="s">
         <v>182</v>
       </c>
-      <c r="B105" s="143"/>
-      <c r="C105" s="144"/>
-      <c r="D105" s="143"/>
-      <c r="E105" s="144"/>
-      <c r="F105" s="144"/>
-      <c r="G105" s="144"/>
-      <c r="H105" s="145"/>
+      <c r="B105" s="191"/>
+      <c r="C105" s="192"/>
+      <c r="D105" s="191"/>
+      <c r="E105" s="192"/>
+      <c r="F105" s="192"/>
+      <c r="G105" s="192"/>
+      <c r="H105" s="129"/>
       <c r="I105" s="71"/>
       <c r="J105" s="25"/>
       <c r="K105" s="26"/>
@@ -6217,16 +6219,16 @@
       <c r="Z105" s="26"/>
     </row>
     <row r="106" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="129" t="s">
+      <c r="A106" s="193" t="s">
         <v>158</v>
       </c>
-      <c r="B106" s="130"/>
-      <c r="C106" s="131"/>
-      <c r="D106" s="130"/>
-      <c r="E106" s="131"/>
-      <c r="F106" s="131"/>
-      <c r="G106" s="131"/>
-      <c r="H106" s="132"/>
+      <c r="B106" s="148"/>
+      <c r="C106" s="149"/>
+      <c r="D106" s="148"/>
+      <c r="E106" s="149"/>
+      <c r="F106" s="149"/>
+      <c r="G106" s="149"/>
+      <c r="H106" s="150"/>
       <c r="I106" s="71"/>
       <c r="J106" s="25"/>
       <c r="K106" s="26"/>
@@ -6483,14 +6485,14 @@
       <c r="Z112" s="26"/>
     </row>
     <row r="113" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="146"/>
-      <c r="B113" s="130"/>
-      <c r="C113" s="131"/>
-      <c r="D113" s="130"/>
-      <c r="E113" s="131"/>
-      <c r="F113" s="131"/>
-      <c r="G113" s="131"/>
-      <c r="H113" s="132"/>
+      <c r="A113" s="194"/>
+      <c r="B113" s="148"/>
+      <c r="C113" s="149"/>
+      <c r="D113" s="148"/>
+      <c r="E113" s="149"/>
+      <c r="F113" s="149"/>
+      <c r="G113" s="149"/>
+      <c r="H113" s="150"/>
       <c r="I113" s="71"/>
       <c r="J113" s="25"/>
       <c r="K113" s="26"/>
@@ -6511,16 +6513,16 @@
       <c r="Z113" s="26"/>
     </row>
     <row r="114" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="125" t="s">
+      <c r="A114" s="161" t="s">
         <v>165</v>
       </c>
-      <c r="B114" s="126"/>
-      <c r="C114" s="127"/>
-      <c r="D114" s="126"/>
-      <c r="E114" s="127"/>
-      <c r="F114" s="127"/>
-      <c r="G114" s="127"/>
-      <c r="H114" s="128"/>
+      <c r="B114" s="131"/>
+      <c r="C114" s="132"/>
+      <c r="D114" s="131"/>
+      <c r="E114" s="132"/>
+      <c r="F114" s="132"/>
+      <c r="G114" s="132"/>
+      <c r="H114" s="133"/>
       <c r="I114" s="71"/>
       <c r="J114" s="25"/>
       <c r="K114" s="26"/>
@@ -7197,16 +7199,16 @@
       <c r="Z130" s="26"/>
     </row>
     <row r="131" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="129" t="s">
+      <c r="A131" s="193" t="s">
         <v>168</v>
       </c>
-      <c r="B131" s="130"/>
-      <c r="C131" s="131"/>
-      <c r="D131" s="130"/>
-      <c r="E131" s="131"/>
-      <c r="F131" s="131"/>
-      <c r="G131" s="131"/>
-      <c r="H131" s="132"/>
+      <c r="B131" s="148"/>
+      <c r="C131" s="149"/>
+      <c r="D131" s="148"/>
+      <c r="E131" s="149"/>
+      <c r="F131" s="149"/>
+      <c r="G131" s="149"/>
+      <c r="H131" s="150"/>
       <c r="I131" s="71"/>
       <c r="J131" s="25"/>
       <c r="K131" s="26"/>
@@ -7242,11 +7244,11 @@
         <v>0</v>
       </c>
       <c r="G132" s="55">
-        <f t="shared" ref="G132:G147" si="4">SUM(E132:F132)</f>
+        <f t="shared" ref="G132:G145" si="4">SUM(E132:F132)</f>
         <v>4</v>
       </c>
       <c r="H132" s="43">
-        <f t="shared" ref="H132:H147" si="5">E132*15+F132*30</f>
+        <f t="shared" ref="H132:H145" si="5">E132*15+F132*30</f>
         <v>60</v>
       </c>
       <c r="I132" s="71"/>
@@ -7270,20 +7272,20 @@
     </row>
     <row r="133" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="13" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B133" s="79" t="s">
-        <v>9</v>
-      </c>
-      <c r="C133" s="55"/>
-      <c r="D133" s="35"/>
-      <c r="E133" s="55">
+        <v>11</v>
+      </c>
+      <c r="C133" s="81"/>
+      <c r="D133" s="82"/>
+      <c r="E133" s="81">
         <v>4</v>
       </c>
-      <c r="F133" s="55">
+      <c r="F133" s="81">
         <v>0</v>
       </c>
-      <c r="G133" s="55">
+      <c r="G133" s="42">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
@@ -7312,10 +7314,10 @@
     </row>
     <row r="134" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B134" s="79" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C134" s="81"/>
       <c r="D134" s="82"/>
@@ -7354,10 +7356,10 @@
     </row>
     <row r="135" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="13" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B135" s="79" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C135" s="81"/>
       <c r="D135" s="82"/>
@@ -7396,10 +7398,10 @@
     </row>
     <row r="136" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="13" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B136" s="79" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C136" s="81"/>
       <c r="D136" s="82"/>
@@ -7437,11 +7439,11 @@
       <c r="Z136" s="26"/>
     </row>
     <row r="137" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="13" t="s">
-        <v>16</v>
+      <c r="A137" s="13">
+        <v>323150</v>
       </c>
       <c r="B137" s="79" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C137" s="81"/>
       <c r="D137" s="82"/>
@@ -7479,11 +7481,11 @@
       <c r="Z137" s="26"/>
     </row>
     <row r="138" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="13">
-        <v>323150</v>
+      <c r="A138" s="13" t="s">
+        <v>20</v>
       </c>
       <c r="B138" s="79" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C138" s="81"/>
       <c r="D138" s="82"/>
@@ -7521,11 +7523,11 @@
       <c r="Z138" s="26"/>
     </row>
     <row r="139" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="13" t="s">
-        <v>20</v>
+      <c r="A139" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="B139" s="79" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C139" s="81"/>
       <c r="D139" s="82"/>
@@ -7563,14 +7565,14 @@
       <c r="Z139" s="26"/>
     </row>
     <row r="140" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="15" t="s">
-        <v>22</v>
+      <c r="A140" s="13" t="s">
+        <v>24</v>
       </c>
       <c r="B140" s="79" t="s">
-        <v>23</v>
-      </c>
-      <c r="C140" s="81"/>
-      <c r="D140" s="82"/>
+        <v>25</v>
+      </c>
+      <c r="C140" s="94"/>
+      <c r="D140" s="95"/>
       <c r="E140" s="81">
         <v>4</v>
       </c>
@@ -7606,14 +7608,14 @@
     </row>
     <row r="141" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B141" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="C141" s="94"/>
-      <c r="D141" s="95"/>
-      <c r="E141" s="81">
+        <v>26</v>
+      </c>
+      <c r="B141" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C141" s="58"/>
+      <c r="D141" s="57"/>
+      <c r="E141" s="96">
         <v>4</v>
       </c>
       <c r="F141" s="81">
@@ -7647,18 +7649,18 @@
       <c r="Z141" s="26"/>
     </row>
     <row r="142" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B142" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C142" s="58"/>
-      <c r="D142" s="57"/>
-      <c r="E142" s="96">
+      <c r="A142" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B142" s="79" t="s">
+        <v>32</v>
+      </c>
+      <c r="C142" s="42"/>
+      <c r="D142" s="41"/>
+      <c r="E142" s="42">
         <v>4</v>
       </c>
-      <c r="F142" s="81">
+      <c r="F142" s="42">
         <v>0</v>
       </c>
       <c r="G142" s="42">
@@ -7690,17 +7692,17 @@
     </row>
     <row r="143" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="13" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B143" s="79" t="s">
-        <v>29</v>
-      </c>
-      <c r="C143" s="90"/>
-      <c r="D143" s="97"/>
-      <c r="E143" s="94">
+        <v>34</v>
+      </c>
+      <c r="C143" s="84"/>
+      <c r="D143" s="85"/>
+      <c r="E143" s="84">
         <v>4</v>
       </c>
-      <c r="F143" s="94">
+      <c r="F143" s="84">
         <v>0</v>
       </c>
       <c r="G143" s="42">
@@ -7731,18 +7733,18 @@
       <c r="Z143" s="26"/>
     </row>
     <row r="144" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="16" t="s">
-        <v>31</v>
+      <c r="A144" s="13" t="s">
+        <v>36</v>
       </c>
       <c r="B144" s="79" t="s">
-        <v>32</v>
-      </c>
-      <c r="C144" s="42"/>
-      <c r="D144" s="41"/>
-      <c r="E144" s="42">
+        <v>37</v>
+      </c>
+      <c r="C144" s="84"/>
+      <c r="D144" s="85"/>
+      <c r="E144" s="84">
         <v>4</v>
       </c>
-      <c r="F144" s="42">
+      <c r="F144" s="84">
         <v>0</v>
       </c>
       <c r="G144" s="42">
@@ -7774,10 +7776,10 @@
     </row>
     <row r="145" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="13" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B145" s="79" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C145" s="84"/>
       <c r="D145" s="85"/>
@@ -7815,28 +7817,14 @@
       <c r="Z145" s="26"/>
     </row>
     <row r="146" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B146" s="79" t="s">
-        <v>37</v>
-      </c>
-      <c r="C146" s="84"/>
-      <c r="D146" s="85"/>
-      <c r="E146" s="84">
-        <v>4</v>
-      </c>
-      <c r="F146" s="84">
-        <v>0</v>
-      </c>
-      <c r="G146" s="42">
-        <f t="shared" si="4"/>
-        <v>4</v>
-      </c>
-      <c r="H146" s="43">
-        <f t="shared" si="5"/>
-        <v>60</v>
-      </c>
+      <c r="A146" s="134"/>
+      <c r="B146" s="131"/>
+      <c r="C146" s="132"/>
+      <c r="D146" s="131"/>
+      <c r="E146" s="132"/>
+      <c r="F146" s="132"/>
+      <c r="G146" s="132"/>
+      <c r="H146" s="133"/>
       <c r="I146" s="71"/>
       <c r="J146" s="25"/>
       <c r="K146" s="26"/>
@@ -7856,29 +7844,17 @@
       <c r="Y146" s="26"/>
       <c r="Z146" s="26"/>
     </row>
-    <row r="147" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B147" s="79" t="s">
-        <v>39</v>
-      </c>
-      <c r="C147" s="84"/>
-      <c r="D147" s="85"/>
-      <c r="E147" s="84">
-        <v>4</v>
-      </c>
-      <c r="F147" s="84">
-        <v>0</v>
-      </c>
-      <c r="G147" s="42">
-        <f t="shared" si="4"/>
-        <v>4</v>
-      </c>
-      <c r="H147" s="43">
-        <f t="shared" si="5"/>
-        <v>60</v>
-      </c>
+    <row r="147" spans="1:26" ht="216" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="159" t="s">
+        <v>214</v>
+      </c>
+      <c r="B147" s="131"/>
+      <c r="C147" s="132"/>
+      <c r="D147" s="131"/>
+      <c r="E147" s="132"/>
+      <c r="F147" s="132"/>
+      <c r="G147" s="132"/>
+      <c r="H147" s="133"/>
       <c r="I147" s="71"/>
       <c r="J147" s="25"/>
       <c r="K147" s="26"/>
@@ -7899,14 +7875,14 @@
       <c r="Z147" s="26"/>
     </row>
     <row r="148" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="133"/>
-      <c r="B148" s="126"/>
-      <c r="C148" s="127"/>
-      <c r="D148" s="126"/>
-      <c r="E148" s="127"/>
-      <c r="F148" s="127"/>
-      <c r="G148" s="127"/>
-      <c r="H148" s="128"/>
+      <c r="A148" s="130"/>
+      <c r="B148" s="131"/>
+      <c r="C148" s="132"/>
+      <c r="D148" s="131"/>
+      <c r="E148" s="132"/>
+      <c r="F148" s="132"/>
+      <c r="G148" s="132"/>
+      <c r="H148" s="133"/>
       <c r="I148" s="71"/>
       <c r="J148" s="25"/>
       <c r="K148" s="26"/>
@@ -7926,17 +7902,15 @@
       <c r="Y148" s="26"/>
       <c r="Z148" s="26"/>
     </row>
-    <row r="149" spans="1:26" ht="127.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="134" t="s">
-        <v>190</v>
-      </c>
-      <c r="B149" s="126"/>
-      <c r="C149" s="127"/>
-      <c r="D149" s="126"/>
-      <c r="E149" s="127"/>
-      <c r="F149" s="127"/>
-      <c r="G149" s="127"/>
-      <c r="H149" s="128"/>
+    <row r="149" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="71"/>
+      <c r="B149" s="25"/>
+      <c r="C149" s="71"/>
+      <c r="D149" s="25"/>
+      <c r="E149" s="71"/>
+      <c r="F149" s="71"/>
+      <c r="G149" s="71"/>
+      <c r="H149" s="71"/>
       <c r="I149" s="71"/>
       <c r="J149" s="25"/>
       <c r="K149" s="26"/>
@@ -7957,14 +7931,14 @@
       <c r="Z149" s="26"/>
     </row>
     <row r="150" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="135"/>
-      <c r="B150" s="126"/>
-      <c r="C150" s="127"/>
-      <c r="D150" s="126"/>
-      <c r="E150" s="127"/>
-      <c r="F150" s="127"/>
-      <c r="G150" s="127"/>
-      <c r="H150" s="128"/>
+      <c r="A150" s="71"/>
+      <c r="B150" s="25"/>
+      <c r="C150" s="71"/>
+      <c r="D150" s="25"/>
+      <c r="E150" s="71"/>
+      <c r="F150" s="71"/>
+      <c r="G150" s="71"/>
+      <c r="H150" s="71"/>
       <c r="I150" s="71"/>
       <c r="J150" s="25"/>
       <c r="K150" s="26"/>
@@ -13500,7 +13474,7 @@
       <c r="Y347" s="26"/>
       <c r="Z347" s="26"/>
     </row>
-    <row r="348" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A348" s="71"/>
       <c r="B348" s="25"/>
       <c r="C348" s="71"/>
@@ -13528,7 +13502,7 @@
       <c r="Y348" s="26"/>
       <c r="Z348" s="26"/>
     </row>
-    <row r="349" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A349" s="71"/>
       <c r="B349" s="25"/>
       <c r="C349" s="71"/>
@@ -31448,69 +31422,68 @@
       <c r="Y988" s="26"/>
       <c r="Z988" s="26"/>
     </row>
-    <row r="989" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A989" s="71"/>
-      <c r="B989" s="25"/>
-      <c r="C989" s="71"/>
-      <c r="D989" s="25"/>
-      <c r="E989" s="71"/>
-      <c r="F989" s="71"/>
-      <c r="G989" s="71"/>
-      <c r="H989" s="71"/>
-      <c r="I989" s="71"/>
-      <c r="J989" s="25"/>
-      <c r="K989" s="26"/>
-      <c r="L989" s="26"/>
-      <c r="M989" s="26"/>
-      <c r="N989" s="27"/>
-      <c r="O989" s="27"/>
-      <c r="P989" s="26"/>
-      <c r="Q989" s="26"/>
-      <c r="R989" s="26"/>
-      <c r="S989" s="26"/>
-      <c r="T989" s="26"/>
-      <c r="U989" s="26"/>
-      <c r="V989" s="26"/>
-      <c r="W989" s="26"/>
-      <c r="X989" s="26"/>
-      <c r="Y989" s="26"/>
-      <c r="Z989" s="26"/>
-    </row>
-    <row r="990" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A990" s="71"/>
-      <c r="B990" s="25"/>
-      <c r="C990" s="71"/>
-      <c r="D990" s="25"/>
-      <c r="E990" s="71"/>
-      <c r="F990" s="71"/>
-      <c r="G990" s="71"/>
-      <c r="H990" s="71"/>
-      <c r="I990" s="71"/>
-      <c r="J990" s="25"/>
-      <c r="K990" s="26"/>
-      <c r="L990" s="26"/>
-      <c r="M990" s="26"/>
-      <c r="N990" s="27"/>
-      <c r="O990" s="27"/>
-      <c r="P990" s="26"/>
-      <c r="Q990" s="26"/>
-      <c r="R990" s="26"/>
-      <c r="S990" s="26"/>
-      <c r="T990" s="26"/>
-      <c r="U990" s="26"/>
-      <c r="V990" s="26"/>
-      <c r="W990" s="26"/>
-      <c r="X990" s="26"/>
-      <c r="Y990" s="26"/>
-      <c r="Z990" s="26"/>
-    </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="A114:H114"/>
+    <mergeCell ref="A131:H131"/>
+    <mergeCell ref="A146:H146"/>
+    <mergeCell ref="A147:H147"/>
+    <mergeCell ref="A148:H148"/>
+    <mergeCell ref="B103:D103"/>
+    <mergeCell ref="F103:H103"/>
+    <mergeCell ref="A105:H105"/>
+    <mergeCell ref="A106:H106"/>
+    <mergeCell ref="A113:H113"/>
+    <mergeCell ref="K100:L100"/>
+    <mergeCell ref="C101:D101"/>
+    <mergeCell ref="F101:H101"/>
+    <mergeCell ref="K101:L101"/>
+    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="F102:H102"/>
+    <mergeCell ref="A97:I97"/>
+    <mergeCell ref="A98:I98"/>
+    <mergeCell ref="A99:I99"/>
+    <mergeCell ref="C100:D100"/>
+    <mergeCell ref="F100:H100"/>
+    <mergeCell ref="B86:D86"/>
+    <mergeCell ref="A88:I88"/>
+    <mergeCell ref="B94:D94"/>
+    <mergeCell ref="A95:I95"/>
+    <mergeCell ref="A96:I96"/>
+    <mergeCell ref="A64:I64"/>
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="A72:I72"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="A81:I81"/>
+    <mergeCell ref="A48:I48"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:H46"/>
+    <mergeCell ref="I46:I47"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:H28"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="B26:D26"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="A9:I9"/>
@@ -31520,68 +31493,14 @@
     <mergeCell ref="E10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="A27:I27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:H28"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A38:I38"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="A45:I45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:H46"/>
-    <mergeCell ref="I46:I47"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:I48"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="A55:I55"/>
-    <mergeCell ref="A56:I56"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="A64:I64"/>
-    <mergeCell ref="B70:D70"/>
-    <mergeCell ref="A72:I72"/>
-    <mergeCell ref="B79:D79"/>
-    <mergeCell ref="A81:I81"/>
-    <mergeCell ref="B86:D86"/>
-    <mergeCell ref="A88:I88"/>
-    <mergeCell ref="B94:D94"/>
-    <mergeCell ref="A95:I95"/>
-    <mergeCell ref="A96:I96"/>
-    <mergeCell ref="A97:I97"/>
-    <mergeCell ref="A98:I98"/>
-    <mergeCell ref="A99:I99"/>
-    <mergeCell ref="C100:D100"/>
-    <mergeCell ref="F100:H100"/>
-    <mergeCell ref="K100:L100"/>
-    <mergeCell ref="C101:D101"/>
-    <mergeCell ref="F101:H101"/>
-    <mergeCell ref="K101:L101"/>
-    <mergeCell ref="C102:D102"/>
-    <mergeCell ref="F102:H102"/>
-    <mergeCell ref="B103:D103"/>
-    <mergeCell ref="F103:H103"/>
-    <mergeCell ref="A105:H105"/>
-    <mergeCell ref="A106:H106"/>
-    <mergeCell ref="A113:H113"/>
-    <mergeCell ref="A114:H114"/>
-    <mergeCell ref="A131:H131"/>
-    <mergeCell ref="A148:H148"/>
-    <mergeCell ref="A149:H149"/>
-    <mergeCell ref="A150:H150"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="F5:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>